<commit_message>
fix: emit custom numFmt definitions in stream exports
</commit_message>
<xml_diff>
--- a/packages/typed-xlsx/examples/financial-report-stream.xlsx
+++ b/packages/typed-xlsx/examples/financial-report-stream.xlsx
@@ -8,138 +8,136 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="40">
   <si>
     <t>2023-03</t>
   </si>
   <si>
+    <t>Sales</t>
+  </si>
+  <si>
+    <t>55.53%</t>
+  </si>
+  <si>
+    <t>88.81%</t>
+  </si>
+  <si>
+    <t>43.71%</t>
+  </si>
+  <si>
+    <t>2023-01</t>
+  </si>
+  <si>
+    <t>Marketing</t>
+  </si>
+  <si>
+    <t>-128.6%</t>
+  </si>
+  <si>
+    <t>-107.63%</t>
+  </si>
+  <si>
+    <t>83.44%</t>
+  </si>
+  <si>
+    <t>19.94%</t>
+  </si>
+  <si>
     <t>Human Resources</t>
   </si>
   <si>
-    <t>82.4%</t>
+    <t>14.74%</t>
+  </si>
+  <si>
+    <t>56.96%</t>
+  </si>
+  <si>
+    <t>88.26%</t>
+  </si>
+  <si>
+    <t>63.3%</t>
+  </si>
+  <si>
+    <t>55.14%</t>
+  </si>
+  <si>
+    <t>2023-10</t>
   </si>
   <si>
     <t>R&amp;D</t>
   </si>
   <si>
-    <t>49.39%</t>
-  </si>
-  <si>
-    <t>Marketing</t>
-  </si>
-  <si>
-    <t>29.1%</t>
-  </si>
-  <si>
-    <t>2023-04</t>
-  </si>
-  <si>
-    <t>-100.1%</t>
-  </si>
-  <si>
-    <t>Sales</t>
-  </si>
-  <si>
-    <t>79.11%</t>
-  </si>
-  <si>
-    <t>-0.54%</t>
-  </si>
-  <si>
-    <t>2023-09</t>
-  </si>
-  <si>
-    <t>68.39%</t>
-  </si>
-  <si>
-    <t>53.1%</t>
-  </si>
-  <si>
-    <t>33.29%</t>
-  </si>
-  <si>
-    <t>2023-05</t>
-  </si>
-  <si>
-    <t>31.9%</t>
-  </si>
-  <si>
-    <t>-25.09%</t>
+    <t>84.85%</t>
+  </si>
+  <si>
+    <t>-84.71%</t>
+  </si>
+  <si>
+    <t>-225.35%</t>
+  </si>
+  <si>
+    <t>-99.07%</t>
+  </si>
+  <si>
+    <t>64.83%</t>
+  </si>
+  <si>
+    <t>59.8%</t>
+  </si>
+  <si>
+    <t>2023-11</t>
+  </si>
+  <si>
+    <t>75.79%</t>
+  </si>
+  <si>
+    <t>-55.02%</t>
+  </si>
+  <si>
+    <t>75.5%</t>
+  </si>
+  <si>
+    <t>2023-06</t>
+  </si>
+  <si>
+    <t>81.56%</t>
+  </si>
+  <si>
+    <t>87.42%</t>
+  </si>
+  <si>
+    <t>68.12%</t>
   </si>
   <si>
     <t>Customer Support</t>
   </si>
   <si>
-    <t>91.77%</t>
-  </si>
-  <si>
-    <t>2023-07</t>
-  </si>
-  <si>
-    <t>82.26%</t>
-  </si>
-  <si>
-    <t>91.73%</t>
-  </si>
-  <si>
-    <t>43.5%</t>
-  </si>
-  <si>
-    <t>2023-12</t>
-  </si>
-  <si>
-    <t>14.24%</t>
-  </si>
-  <si>
-    <t>88.04%</t>
-  </si>
-  <si>
-    <t>-4.16%</t>
-  </si>
-  <si>
-    <t>2023-01</t>
-  </si>
-  <si>
-    <t>86.2%</t>
-  </si>
-  <si>
-    <t>92.42%</t>
-  </si>
-  <si>
-    <t>-0.41%</t>
-  </si>
-  <si>
-    <t>-163.02%</t>
-  </si>
-  <si>
-    <t>17.26%</t>
-  </si>
-  <si>
-    <t>17.35%</t>
-  </si>
-  <si>
-    <t>-18.4%</t>
-  </si>
-  <si>
-    <t>45.72%</t>
-  </si>
-  <si>
-    <t>60.8%</t>
-  </si>
-  <si>
-    <t>73.53%</t>
-  </si>
-  <si>
-    <t>49.92%</t>
-  </si>
-  <si>
-    <t>41.28%</t>
+    <t>38.36%</t>
+  </si>
+  <si>
+    <t>52.04%</t>
+  </si>
+  <si>
+    <t>82.74%</t>
+  </si>
+  <si>
+    <t>-223.57%</t>
+  </si>
+  <si>
+    <t>89.93%</t>
+  </si>
+  <si>
+    <t>-17.67%</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="$#,##0.00"/>
+    <numFmt numFmtId="165" formatCode="0.00&quot;%&quot;"/>
+  </numFmts>
   <fonts count="5">
     <font>
       <sz val="11"/>
@@ -343,46 +341,46 @@
         <v>1</v>
       </c>
       <c r="C2" s="2">
-        <v>87597</v>
+        <v>76484</v>
       </c>
       <c r="D2" s="2">
-        <v>15420</v>
+        <v>34009</v>
       </c>
       <c r="E2" s="3">
-        <v>72177</v>
+        <v>42475</v>
       </c>
       <c r="F2" s="4" t="s">
         <v>2</v>
       </c>
       <c r="G2" s="2">
-        <v>173654</v>
+        <v>199568</v>
       </c>
       <c r="H2" s="2">
-        <v>69480</v>
+        <v>68564</v>
       </c>
       <c r="I2" s="3">
-        <v>104174</v>
+        <v>131004</v>
       </c>
       <c r="J2" s="5">
-        <v>53.63</v>
+        <v>62.68333333333334</v>
       </c>
     </row>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="1"/>
       <c r="B3" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" s="2">
+        <v>77005</v>
+      </c>
+      <c r="D3" s="2">
+        <v>8618</v>
+      </c>
+      <c r="E3" s="3">
+        <v>68387</v>
+      </c>
+      <c r="F3" s="4" t="s">
         <v>3</v>
-      </c>
-      <c r="C3" s="2">
-        <v>34259</v>
-      </c>
-      <c r="D3" s="2">
-        <v>17337</v>
-      </c>
-      <c r="E3" s="3">
-        <v>16922</v>
-      </c>
-      <c r="F3" s="4" t="s">
-        <v>4</v>
       </c>
       <c r="G3" s="2"/>
       <c r="H3" s="2"/>
@@ -392,19 +390,19 @@
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="1"/>
       <c r="B4" s="1" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C4" s="2">
-        <v>51798</v>
+        <v>46079</v>
       </c>
       <c r="D4" s="2">
-        <v>36723</v>
+        <v>25937</v>
       </c>
       <c r="E4" s="3">
-        <v>15075</v>
+        <v>20142</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="G4" s="2"/>
       <c r="H4" s="2"/>
@@ -413,128 +411,128 @@
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5" s="2">
+        <v>15429</v>
+      </c>
+      <c r="D5" s="2">
+        <v>35271</v>
+      </c>
+      <c r="E5" s="6">
+        <v>-19842</v>
+      </c>
+      <c r="F5" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C5" s="2">
-        <v>12566</v>
-      </c>
-      <c r="D5" s="2">
-        <v>25145</v>
-      </c>
-      <c r="E5" s="6">
-        <v>-12579</v>
-      </c>
-      <c r="F5" s="7" t="s">
-        <v>8</v>
-      </c>
       <c r="G5" s="2">
-        <v>112251</v>
+        <v>79811</v>
       </c>
       <c r="H5" s="2">
-        <v>62061</v>
-      </c>
-      <c r="I5" s="3">
-        <v>50190</v>
+        <v>84501</v>
+      </c>
+      <c r="I5" s="6">
+        <v>-4690</v>
       </c>
       <c r="J5" s="8">
-        <v>-7.176666666666665</v>
+        <v>-50.93</v>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="1"/>
       <c r="B6" s="1" t="s">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="C6" s="2">
-        <v>79479</v>
+        <v>20186</v>
       </c>
       <c r="D6" s="2">
-        <v>16601</v>
-      </c>
-      <c r="E6" s="3">
-        <v>62878</v>
-      </c>
-      <c r="F6" s="4" t="s">
-        <v>10</v>
+        <v>41912</v>
+      </c>
+      <c r="E6" s="6">
+        <v>-21726</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>8</v>
       </c>
       <c r="G6" s="2"/>
       <c r="H6" s="2"/>
-      <c r="I6" s="3"/>
+      <c r="I6" s="6"/>
       <c r="J6" s="8"/>
     </row>
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="1"/>
       <c r="B7" s="1" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C7" s="2">
-        <v>20206</v>
+        <v>44196</v>
       </c>
       <c r="D7" s="2">
-        <v>20315</v>
-      </c>
-      <c r="E7" s="6">
-        <v>-109</v>
-      </c>
-      <c r="F7" s="7" t="s">
-        <v>11</v>
+        <v>7318</v>
+      </c>
+      <c r="E7" s="3">
+        <v>36878</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>9</v>
       </c>
       <c r="G7" s="2"/>
       <c r="H7" s="2"/>
-      <c r="I7" s="3"/>
+      <c r="I7" s="6"/>
       <c r="J7" s="8"/>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="1" t="s">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C8" s="2">
-        <v>96110</v>
+        <v>42485</v>
       </c>
       <c r="D8" s="2">
-        <v>30379</v>
+        <v>34014</v>
       </c>
       <c r="E8" s="3">
-        <v>65731</v>
+        <v>8471</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="G8" s="2">
-        <v>257029</v>
+        <v>151315</v>
       </c>
       <c r="H8" s="2">
-        <v>120402</v>
+        <v>94383</v>
       </c>
       <c r="I8" s="3">
-        <v>136627</v>
+        <v>56932</v>
       </c>
       <c r="J8" s="5">
-        <v>51.593333333333334</v>
+        <v>30.546666666666667</v>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="1"/>
       <c r="B9" s="1" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C9" s="2">
-        <v>87446</v>
+        <v>32032</v>
       </c>
       <c r="D9" s="2">
-        <v>41012</v>
+        <v>27312</v>
       </c>
       <c r="E9" s="3">
-        <v>46434</v>
+        <v>4720</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="G9" s="2"/>
       <c r="H9" s="2"/>
@@ -544,19 +542,19 @@
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="1"/>
       <c r="B10" s="1" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C10" s="2">
-        <v>73473</v>
+        <v>76798</v>
       </c>
       <c r="D10" s="2">
-        <v>49011</v>
+        <v>33057</v>
       </c>
       <c r="E10" s="3">
-        <v>24462</v>
+        <v>43741</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="G10" s="2"/>
       <c r="H10" s="2"/>
@@ -565,52 +563,52 @@
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="1" t="s">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C11" s="2">
-        <v>72867</v>
+        <v>46186</v>
       </c>
       <c r="D11" s="2">
-        <v>49620</v>
+        <v>5421</v>
       </c>
       <c r="E11" s="3">
-        <v>23247</v>
+        <v>40765</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="G11" s="2">
-        <v>200022</v>
+        <v>194665</v>
       </c>
       <c r="H11" s="2">
-        <v>102384</v>
+        <v>64052</v>
       </c>
       <c r="I11" s="3">
-        <v>97638</v>
+        <v>130613</v>
       </c>
       <c r="J11" s="5">
-        <v>32.86</v>
+        <v>68.89999999999999</v>
       </c>
     </row>
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="1"/>
       <c r="B12" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C12" s="2">
-        <v>36193</v>
+        <v>97804</v>
       </c>
       <c r="D12" s="2">
-        <v>45274</v>
-      </c>
-      <c r="E12" s="6">
-        <v>-9081</v>
-      </c>
-      <c r="F12" s="7" t="s">
-        <v>18</v>
+        <v>35896</v>
+      </c>
+      <c r="E12" s="3">
+        <v>61908</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>15</v>
       </c>
       <c r="G12" s="2"/>
       <c r="H12" s="2"/>
@@ -620,19 +618,19 @@
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="1"/>
       <c r="B13" s="1" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="C13" s="2">
-        <v>90962</v>
+        <v>50675</v>
       </c>
       <c r="D13" s="2">
-        <v>7490</v>
+        <v>22735</v>
       </c>
       <c r="E13" s="3">
-        <v>83472</v>
+        <v>27940</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="G13" s="2"/>
       <c r="H13" s="2"/>
@@ -641,57 +639,57 @@
     </row>
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="1" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B14" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C14" s="2">
+        <v>63533</v>
+      </c>
+      <c r="D14" s="2">
+        <v>9623</v>
+      </c>
+      <c r="E14" s="3">
+        <v>53910</v>
+      </c>
+      <c r="F14" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="C14" s="2">
-        <v>70739</v>
-      </c>
-      <c r="D14" s="2">
-        <v>12549</v>
-      </c>
-      <c r="E14" s="3">
-        <v>58190</v>
-      </c>
-      <c r="F14" s="4" t="s">
-        <v>22</v>
-      </c>
       <c r="G14" s="2">
-        <v>232090</v>
+        <v>100260</v>
       </c>
       <c r="H14" s="2">
-        <v>59008</v>
+        <v>92780</v>
       </c>
       <c r="I14" s="3">
-        <v>173082</v>
-      </c>
-      <c r="J14" s="5">
-        <v>72.49666666666667</v>
+        <v>7480</v>
+      </c>
+      <c r="J14" s="8">
+        <v>-75.07</v>
       </c>
     </row>
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="1"/>
       <c r="B15" s="1" t="s">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="C15" s="2">
-        <v>92675</v>
+        <v>25834</v>
       </c>
       <c r="D15" s="2">
-        <v>7660</v>
-      </c>
-      <c r="E15" s="3">
-        <v>85015</v>
-      </c>
-      <c r="F15" s="4" t="s">
-        <v>23</v>
+        <v>47717</v>
+      </c>
+      <c r="E15" s="6">
+        <v>-21883</v>
+      </c>
+      <c r="F15" s="7" t="s">
+        <v>20</v>
       </c>
       <c r="G15" s="2"/>
       <c r="H15" s="2"/>
       <c r="I15" s="3"/>
-      <c r="J15" s="5"/>
+      <c r="J15" s="8"/>
     </row>
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="1"/>
@@ -699,70 +697,70 @@
         <v>1</v>
       </c>
       <c r="C16" s="2">
-        <v>68676</v>
+        <v>10893</v>
       </c>
       <c r="D16" s="2">
-        <v>38799</v>
-      </c>
-      <c r="E16" s="3">
-        <v>29877</v>
-      </c>
-      <c r="F16" s="4" t="s">
-        <v>24</v>
+        <v>35440</v>
+      </c>
+      <c r="E16" s="6">
+        <v>-24547</v>
+      </c>
+      <c r="F16" s="7" t="s">
+        <v>21</v>
       </c>
       <c r="G16" s="2"/>
       <c r="H16" s="2"/>
       <c r="I16" s="3"/>
-      <c r="J16" s="5"/>
+      <c r="J16" s="8"/>
     </row>
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="1" t="s">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C17" s="2">
-        <v>47863</v>
+        <v>16716</v>
       </c>
       <c r="D17" s="2">
-        <v>41049</v>
-      </c>
-      <c r="E17" s="3">
-        <v>6814</v>
-      </c>
-      <c r="F17" s="4" t="s">
-        <v>26</v>
+        <v>33276</v>
+      </c>
+      <c r="E17" s="6">
+        <v>-16560</v>
+      </c>
+      <c r="F17" s="7" t="s">
+        <v>22</v>
       </c>
       <c r="G17" s="2">
-        <v>166557</v>
+        <v>173285</v>
       </c>
       <c r="H17" s="2">
-        <v>98843</v>
+        <v>92420</v>
       </c>
       <c r="I17" s="3">
-        <v>67714</v>
+        <v>80865</v>
       </c>
       <c r="J17" s="5">
-        <v>32.70666666666667</v>
+        <v>8.520000000000001</v>
       </c>
     </row>
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="1"/>
       <c r="B18" s="1" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C18" s="2">
-        <v>71410</v>
+        <v>75519</v>
       </c>
       <c r="D18" s="2">
-        <v>8543</v>
+        <v>26559</v>
       </c>
       <c r="E18" s="3">
-        <v>62867</v>
+        <v>48960</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="G18" s="2"/>
       <c r="H18" s="2"/>
@@ -772,19 +770,19 @@
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="1"/>
       <c r="B19" s="1" t="s">
-        <v>3</v>
+        <v>18</v>
       </c>
       <c r="C19" s="2">
-        <v>47284</v>
+        <v>81050</v>
       </c>
       <c r="D19" s="2">
-        <v>49251</v>
-      </c>
-      <c r="E19" s="6">
-        <v>-1967</v>
-      </c>
-      <c r="F19" s="7" t="s">
-        <v>28</v>
+        <v>32585</v>
+      </c>
+      <c r="E19" s="3">
+        <v>48465</v>
+      </c>
+      <c r="F19" s="4" t="s">
+        <v>24</v>
       </c>
       <c r="G19" s="2"/>
       <c r="H19" s="2"/>
@@ -793,52 +791,52 @@
     </row>
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="1" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="C20" s="2">
-        <v>58882</v>
+        <v>72400</v>
       </c>
       <c r="D20" s="2">
-        <v>8127</v>
+        <v>17525</v>
       </c>
       <c r="E20" s="3">
-        <v>50755</v>
+        <v>54875</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="G20" s="2">
-        <v>169803</v>
+        <v>190025</v>
       </c>
       <c r="H20" s="2">
-        <v>30938</v>
+        <v>83570</v>
       </c>
       <c r="I20" s="3">
-        <v>138865</v>
+        <v>106455</v>
       </c>
       <c r="J20" s="5">
-        <v>59.403333333333336</v>
+        <v>32.09</v>
       </c>
     </row>
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="1"/>
       <c r="B21" s="1" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="C21" s="2">
-        <v>95408</v>
+        <v>28523</v>
       </c>
       <c r="D21" s="2">
-        <v>7234</v>
-      </c>
-      <c r="E21" s="3">
-        <v>88174</v>
-      </c>
-      <c r="F21" s="4" t="s">
-        <v>31</v>
+        <v>44216</v>
+      </c>
+      <c r="E21" s="6">
+        <v>-15693</v>
+      </c>
+      <c r="F21" s="7" t="s">
+        <v>27</v>
       </c>
       <c r="G21" s="2"/>
       <c r="H21" s="2"/>
@@ -848,19 +846,19 @@
     <row r="22" ht="30" customHeight="1">
       <c r="A22" s="1"/>
       <c r="B22" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C22" s="2">
-        <v>15513</v>
+        <v>89102</v>
       </c>
       <c r="D22" s="2">
-        <v>15577</v>
-      </c>
-      <c r="E22" s="6">
-        <v>-64</v>
-      </c>
-      <c r="F22" s="7" t="s">
-        <v>32</v>
+        <v>21829</v>
+      </c>
+      <c r="E22" s="3">
+        <v>67273</v>
+      </c>
+      <c r="F22" s="4" t="s">
+        <v>28</v>
       </c>
       <c r="G22" s="2"/>
       <c r="H22" s="2"/>
@@ -869,128 +867,128 @@
     </row>
     <row r="23" ht="30" customHeight="1">
       <c r="A23" s="1" t="s">
-        <v>16</v>
+        <v>29</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="C23" s="2">
-        <v>11806</v>
+        <v>53249</v>
       </c>
       <c r="D23" s="2">
-        <v>31052</v>
-      </c>
-      <c r="E23" s="6">
-        <v>-19246</v>
-      </c>
-      <c r="F23" s="7" t="s">
-        <v>33</v>
+        <v>9820</v>
+      </c>
+      <c r="E23" s="3">
+        <v>43429</v>
+      </c>
+      <c r="F23" s="4" t="s">
+        <v>30</v>
       </c>
       <c r="G23" s="2">
-        <v>78970</v>
+        <v>235161</v>
       </c>
       <c r="H23" s="2">
-        <v>86597</v>
-      </c>
-      <c r="I23" s="6">
-        <v>-7627</v>
-      </c>
-      <c r="J23" s="8">
-        <v>-42.80333333333334</v>
+        <v>49550</v>
+      </c>
+      <c r="I23" s="3">
+        <v>185611</v>
+      </c>
+      <c r="J23" s="5">
+        <v>79.03333333333335</v>
       </c>
     </row>
     <row r="24" ht="30" customHeight="1">
       <c r="A24" s="1"/>
       <c r="B24" s="1" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="C24" s="2">
-        <v>38775</v>
+        <v>94602</v>
       </c>
       <c r="D24" s="2">
-        <v>32082</v>
+        <v>11899</v>
       </c>
       <c r="E24" s="3">
-        <v>6693</v>
+        <v>82703</v>
       </c>
       <c r="F24" s="4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="G24" s="2"/>
       <c r="H24" s="2"/>
-      <c r="I24" s="6"/>
-      <c r="J24" s="8"/>
+      <c r="I24" s="3"/>
+      <c r="J24" s="5"/>
     </row>
     <row r="25" ht="30" customHeight="1">
       <c r="A25" s="1"/>
       <c r="B25" s="1" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="C25" s="2">
-        <v>28389</v>
+        <v>87310</v>
       </c>
       <c r="D25" s="2">
-        <v>23463</v>
+        <v>27831</v>
       </c>
       <c r="E25" s="3">
-        <v>4926</v>
+        <v>59479</v>
       </c>
       <c r="F25" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="G25" s="2"/>
       <c r="H25" s="2"/>
-      <c r="I25" s="6"/>
-      <c r="J25" s="8"/>
+      <c r="I25" s="3"/>
+      <c r="J25" s="5"/>
     </row>
     <row r="26" ht="30" customHeight="1">
       <c r="A26" s="1" t="s">
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>5</v>
+        <v>33</v>
       </c>
       <c r="C26" s="2">
-        <v>23883</v>
+        <v>26292</v>
       </c>
       <c r="D26" s="2">
-        <v>28278</v>
-      </c>
-      <c r="E26" s="6">
-        <v>-4395</v>
-      </c>
-      <c r="F26" s="7" t="s">
-        <v>36</v>
+        <v>16206</v>
+      </c>
+      <c r="E26" s="3">
+        <v>10086</v>
+      </c>
+      <c r="F26" s="4" t="s">
+        <v>34</v>
       </c>
       <c r="G26" s="2">
-        <v>145593</v>
+        <v>140616</v>
       </c>
       <c r="H26" s="2">
-        <v>88811</v>
+        <v>57174</v>
       </c>
       <c r="I26" s="3">
-        <v>56782</v>
+        <v>83442</v>
       </c>
       <c r="J26" s="5">
-        <v>29.373333333333335</v>
+        <v>57.71333333333333</v>
       </c>
     </row>
     <row r="27" ht="30" customHeight="1">
       <c r="A27" s="1"/>
       <c r="B27" s="1" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="C27" s="2">
-        <v>85025</v>
+        <v>69157</v>
       </c>
       <c r="D27" s="2">
-        <v>46154</v>
+        <v>33170</v>
       </c>
       <c r="E27" s="3">
-        <v>38871</v>
+        <v>35987</v>
       </c>
       <c r="F27" s="4" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="G27" s="2"/>
       <c r="H27" s="2"/>
@@ -1000,19 +998,19 @@
     <row r="28" ht="30" customHeight="1">
       <c r="A28" s="1"/>
       <c r="B28" s="1" t="s">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="C28" s="2">
-        <v>36685</v>
+        <v>45167</v>
       </c>
       <c r="D28" s="2">
-        <v>14379</v>
+        <v>7798</v>
       </c>
       <c r="E28" s="3">
-        <v>22306</v>
+        <v>37369</v>
       </c>
       <c r="F28" s="4" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="G28" s="2"/>
       <c r="H28" s="2"/>
@@ -1021,92 +1019,92 @@
     </row>
     <row r="29" ht="30" customHeight="1">
       <c r="A29" s="1" t="s">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C29" s="2">
-        <v>97567</v>
+        <v>10786</v>
       </c>
       <c r="D29" s="2">
-        <v>25825</v>
-      </c>
-      <c r="E29" s="3">
-        <v>71742</v>
-      </c>
-      <c r="F29" s="4" t="s">
-        <v>39</v>
+        <v>34900</v>
+      </c>
+      <c r="E29" s="6">
+        <v>-24114</v>
+      </c>
+      <c r="F29" s="7" t="s">
+        <v>37</v>
       </c>
       <c r="G29" s="2">
-        <v>199934</v>
+        <v>112706</v>
       </c>
       <c r="H29" s="2">
-        <v>79238</v>
+        <v>60191</v>
       </c>
       <c r="I29" s="3">
-        <v>120696</v>
-      </c>
-      <c r="J29" s="5">
-        <v>54.910000000000004</v>
+        <v>52515</v>
+      </c>
+      <c r="J29" s="8">
+        <v>-50.43666666666667</v>
       </c>
     </row>
     <row r="30" ht="30" customHeight="1">
       <c r="A30" s="1"/>
       <c r="B30" s="1" t="s">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C30" s="2">
-        <v>77553</v>
+        <v>87954</v>
       </c>
       <c r="D30" s="2">
-        <v>38841</v>
+        <v>8857</v>
       </c>
       <c r="E30" s="3">
-        <v>38712</v>
+        <v>79097</v>
       </c>
       <c r="F30" s="4" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="G30" s="2"/>
       <c r="H30" s="2"/>
       <c r="I30" s="3"/>
-      <c r="J30" s="5"/>
+      <c r="J30" s="8"/>
     </row>
     <row r="31" ht="30" customHeight="1">
       <c r="A31" s="1"/>
       <c r="B31" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C31" s="2">
-        <v>24814</v>
+        <v>13966</v>
       </c>
       <c r="D31" s="2">
-        <v>14572</v>
-      </c>
-      <c r="E31" s="3">
-        <v>10242</v>
-      </c>
-      <c r="F31" s="4" t="s">
-        <v>41</v>
+        <v>16434</v>
+      </c>
+      <c r="E31" s="6">
+        <v>-2468</v>
+      </c>
+      <c r="F31" s="7" t="s">
+        <v>39</v>
       </c>
       <c r="G31" s="2"/>
       <c r="H31" s="2"/>
       <c r="I31" s="3"/>
-      <c r="J31" s="5"/>
+      <c r="J31" s="8"/>
     </row>
     <row r="32" ht="30" customHeight="1">
       <c r="G32" s="10">
-        <v>1735903</v>
+        <v>1577412</v>
       </c>
       <c r="H32" s="10">
-        <v>797762</v>
+        <v>747185</v>
       </c>
       <c r="I32" s="11">
-        <v>938141</v>
+        <v>830227</v>
       </c>
       <c r="J32" s="12">
-        <v>33.69933333333334</v>
+        <v>16.305000000000003</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(monorepo): add agent rules and refresh examples
</commit_message>
<xml_diff>
--- a/packages/typed-xlsx/examples/financial-report-stream.xlsx
+++ b/packages/typed-xlsx/examples/financial-report-stream.xlsx
@@ -8,126 +8,129 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="41">
+  <si>
+    <t>2023-02</t>
+  </si>
+  <si>
+    <t>Marketing</t>
+  </si>
+  <si>
+    <t>-87.07%</t>
+  </si>
+  <si>
+    <t>Sales</t>
+  </si>
+  <si>
+    <t>-54.41%</t>
+  </si>
+  <si>
+    <t>Customer Support</t>
+  </si>
+  <si>
+    <t>41.25%</t>
+  </si>
+  <si>
+    <t>2023-12</t>
+  </si>
+  <si>
+    <t>54.67%</t>
+  </si>
+  <si>
+    <t>57.8%</t>
+  </si>
+  <si>
+    <t>86.51%</t>
+  </si>
+  <si>
+    <t>2023-06</t>
+  </si>
+  <si>
+    <t>92.22%</t>
+  </si>
+  <si>
+    <t>-50.82%</t>
+  </si>
+  <si>
+    <t>78.61%</t>
+  </si>
+  <si>
+    <t>2023-01</t>
+  </si>
+  <si>
+    <t>R&amp;D</t>
+  </si>
+  <si>
+    <t>89.55%</t>
+  </si>
+  <si>
+    <t>69.8%</t>
+  </si>
+  <si>
+    <t>-184.72%</t>
+  </si>
   <si>
     <t>2023-03</t>
   </si>
   <si>
-    <t>Sales</t>
-  </si>
-  <si>
-    <t>55.53%</t>
-  </si>
-  <si>
-    <t>88.81%</t>
-  </si>
-  <si>
-    <t>43.71%</t>
-  </si>
-  <si>
-    <t>2023-01</t>
-  </si>
-  <si>
-    <t>Marketing</t>
-  </si>
-  <si>
-    <t>-128.6%</t>
-  </si>
-  <si>
-    <t>-107.63%</t>
-  </si>
-  <si>
-    <t>83.44%</t>
-  </si>
-  <si>
-    <t>19.94%</t>
+    <t>43%</t>
   </si>
   <si>
     <t>Human Resources</t>
   </si>
   <si>
-    <t>14.74%</t>
-  </si>
-  <si>
-    <t>56.96%</t>
-  </si>
-  <si>
-    <t>88.26%</t>
-  </si>
-  <si>
-    <t>63.3%</t>
-  </si>
-  <si>
-    <t>55.14%</t>
+    <t>-102.86%</t>
+  </si>
+  <si>
+    <t>71.23%</t>
+  </si>
+  <si>
+    <t>48.54%</t>
+  </si>
+  <si>
+    <t>59.38%</t>
+  </si>
+  <si>
+    <t>26.75%</t>
+  </si>
+  <si>
+    <t>-142.28%</t>
+  </si>
+  <si>
+    <t>49.46%</t>
+  </si>
+  <si>
+    <t>21.44%</t>
+  </si>
+  <si>
+    <t>80.7%</t>
+  </si>
+  <si>
+    <t>79.61%</t>
+  </si>
+  <si>
+    <t>71.79%</t>
   </si>
   <si>
     <t>2023-10</t>
   </si>
   <si>
-    <t>R&amp;D</t>
-  </si>
-  <si>
-    <t>84.85%</t>
-  </si>
-  <si>
-    <t>-84.71%</t>
-  </si>
-  <si>
-    <t>-225.35%</t>
-  </si>
-  <si>
-    <t>-99.07%</t>
-  </si>
-  <si>
-    <t>64.83%</t>
-  </si>
-  <si>
-    <t>59.8%</t>
-  </si>
-  <si>
-    <t>2023-11</t>
-  </si>
-  <si>
-    <t>75.79%</t>
-  </si>
-  <si>
-    <t>-55.02%</t>
-  </si>
-  <si>
-    <t>75.5%</t>
-  </si>
-  <si>
-    <t>2023-06</t>
-  </si>
-  <si>
-    <t>81.56%</t>
-  </si>
-  <si>
-    <t>87.42%</t>
-  </si>
-  <si>
-    <t>68.12%</t>
-  </si>
-  <si>
-    <t>Customer Support</t>
-  </si>
-  <si>
-    <t>38.36%</t>
-  </si>
-  <si>
-    <t>52.04%</t>
-  </si>
-  <si>
-    <t>82.74%</t>
-  </si>
-  <si>
-    <t>-223.57%</t>
-  </si>
-  <si>
-    <t>89.93%</t>
-  </si>
-  <si>
-    <t>-17.67%</t>
+    <t>48.76%</t>
+  </si>
+  <si>
+    <t>29.41%</t>
+  </si>
+  <si>
+    <t>59%</t>
+  </si>
+  <si>
+    <t>47.06%</t>
+  </si>
+  <si>
+    <t>67.98%</t>
+  </si>
+  <si>
+    <t>64.89%</t>
   </si>
 </sst>
 </file>
@@ -144,10 +147,10 @@
       <name val="Calibri"/>
     </font>
     <font>
-      <color rgb="FF007500"/>
+      <color rgb="FFFF0000"/>
     </font>
     <font>
-      <color rgb="FFFF0000"/>
+      <color rgb="FF007500"/>
     </font>
     <font>
       <b/>
@@ -341,46 +344,46 @@
         <v>1</v>
       </c>
       <c r="C2" s="2">
-        <v>76484</v>
+        <v>26542</v>
       </c>
       <c r="D2" s="2">
-        <v>34009</v>
+        <v>49653</v>
       </c>
       <c r="E2" s="3">
-        <v>42475</v>
+        <v>-23111</v>
       </c>
       <c r="F2" s="4" t="s">
         <v>2</v>
       </c>
       <c r="G2" s="2">
-        <v>199568</v>
+        <v>110255</v>
       </c>
       <c r="H2" s="2">
-        <v>68564</v>
+        <v>125998</v>
       </c>
       <c r="I2" s="3">
-        <v>131004</v>
+        <v>-15743</v>
       </c>
       <c r="J2" s="5">
-        <v>62.68333333333334</v>
+        <v>-33.41</v>
       </c>
     </row>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="1"/>
       <c r="B3" s="1" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C3" s="2">
-        <v>77005</v>
+        <v>28398</v>
       </c>
       <c r="D3" s="2">
-        <v>8618</v>
+        <v>43848</v>
       </c>
       <c r="E3" s="3">
-        <v>68387</v>
+        <v>-15450</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G3" s="2"/>
       <c r="H3" s="2"/>
@@ -390,19 +393,19 @@
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="1"/>
       <c r="B4" s="1" t="s">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C4" s="2">
-        <v>46079</v>
+        <v>55315</v>
       </c>
       <c r="D4" s="2">
-        <v>25937</v>
-      </c>
-      <c r="E4" s="3">
-        <v>20142</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>4</v>
+        <v>32497</v>
+      </c>
+      <c r="E4" s="6">
+        <v>22818</v>
+      </c>
+      <c r="F4" s="7" t="s">
+        <v>6</v>
       </c>
       <c r="G4" s="2"/>
       <c r="H4" s="2"/>
@@ -411,52 +414,52 @@
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="1" t="s">
-        <v>6</v>
-      </c>
       <c r="C5" s="2">
-        <v>15429</v>
+        <v>80795</v>
       </c>
       <c r="D5" s="2">
-        <v>35271</v>
+        <v>36626</v>
       </c>
       <c r="E5" s="6">
-        <v>-19842</v>
+        <v>44169</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G5" s="2">
-        <v>79811</v>
+        <v>156044</v>
       </c>
       <c r="H5" s="2">
-        <v>84501</v>
+        <v>55124</v>
       </c>
       <c r="I5" s="6">
-        <v>-4690</v>
+        <v>100920</v>
       </c>
       <c r="J5" s="8">
-        <v>-50.93</v>
+        <v>66.32666666666667</v>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="1"/>
       <c r="B6" s="1" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C6" s="2">
-        <v>20186</v>
+        <v>29071</v>
       </c>
       <c r="D6" s="2">
-        <v>41912</v>
+        <v>12267</v>
       </c>
       <c r="E6" s="6">
-        <v>-21726</v>
+        <v>16804</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G6" s="2"/>
       <c r="H6" s="2"/>
@@ -466,19 +469,19 @@
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="1"/>
       <c r="B7" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C7" s="2">
-        <v>44196</v>
+        <v>46178</v>
       </c>
       <c r="D7" s="2">
-        <v>7318</v>
-      </c>
-      <c r="E7" s="3">
-        <v>36878</v>
-      </c>
-      <c r="F7" s="4" t="s">
-        <v>9</v>
+        <v>6231</v>
+      </c>
+      <c r="E7" s="6">
+        <v>39947</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>10</v>
       </c>
       <c r="G7" s="2"/>
       <c r="H7" s="2"/>
@@ -487,208 +490,208 @@
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="1" t="s">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C8" s="2">
-        <v>42485</v>
+        <v>77643</v>
       </c>
       <c r="D8" s="2">
-        <v>34014</v>
-      </c>
-      <c r="E8" s="3">
-        <v>8471</v>
-      </c>
-      <c r="F8" s="4" t="s">
-        <v>10</v>
+        <v>6038</v>
+      </c>
+      <c r="E8" s="6">
+        <v>71605</v>
+      </c>
+      <c r="F8" s="7" t="s">
+        <v>12</v>
       </c>
       <c r="G8" s="2">
-        <v>151315</v>
+        <v>120670</v>
       </c>
       <c r="H8" s="2">
-        <v>94383</v>
-      </c>
-      <c r="I8" s="3">
-        <v>56932</v>
-      </c>
-      <c r="J8" s="5">
-        <v>30.546666666666667</v>
+        <v>39747</v>
+      </c>
+      <c r="I8" s="6">
+        <v>80923</v>
+      </c>
+      <c r="J8" s="8">
+        <v>40.00333333333333</v>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="1"/>
       <c r="B9" s="1" t="s">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="C9" s="2">
-        <v>32032</v>
+        <v>18933</v>
       </c>
       <c r="D9" s="2">
-        <v>27312</v>
+        <v>28555</v>
       </c>
       <c r="E9" s="3">
-        <v>4720</v>
+        <v>-9622</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G9" s="2"/>
       <c r="H9" s="2"/>
-      <c r="I9" s="3"/>
-      <c r="J9" s="5"/>
+      <c r="I9" s="6"/>
+      <c r="J9" s="8"/>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="1"/>
       <c r="B10" s="1" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C10" s="2">
-        <v>76798</v>
+        <v>24094</v>
       </c>
       <c r="D10" s="2">
-        <v>33057</v>
-      </c>
-      <c r="E10" s="3">
-        <v>43741</v>
-      </c>
-      <c r="F10" s="4" t="s">
-        <v>13</v>
+        <v>5154</v>
+      </c>
+      <c r="E10" s="6">
+        <v>18940</v>
+      </c>
+      <c r="F10" s="7" t="s">
+        <v>14</v>
       </c>
       <c r="G10" s="2"/>
       <c r="H10" s="2"/>
-      <c r="I10" s="3"/>
-      <c r="J10" s="5"/>
+      <c r="I10" s="6"/>
+      <c r="J10" s="8"/>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="1" t="s">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="C11" s="2">
-        <v>46186</v>
+        <v>76041</v>
       </c>
       <c r="D11" s="2">
-        <v>5421</v>
-      </c>
-      <c r="E11" s="3">
-        <v>40765</v>
-      </c>
-      <c r="F11" s="4" t="s">
-        <v>14</v>
+        <v>7943</v>
+      </c>
+      <c r="E11" s="6">
+        <v>68098</v>
+      </c>
+      <c r="F11" s="7" t="s">
+        <v>17</v>
       </c>
       <c r="G11" s="2">
-        <v>194665</v>
+        <v>182960</v>
       </c>
       <c r="H11" s="2">
-        <v>64052</v>
-      </c>
-      <c r="I11" s="3">
-        <v>130613</v>
+        <v>72656</v>
+      </c>
+      <c r="I11" s="6">
+        <v>110304</v>
       </c>
       <c r="J11" s="5">
-        <v>68.89999999999999</v>
+        <v>-8.456666666666669</v>
       </c>
     </row>
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="1"/>
       <c r="B12" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C12" s="2">
-        <v>97804</v>
+        <v>94180</v>
       </c>
       <c r="D12" s="2">
-        <v>35896</v>
-      </c>
-      <c r="E12" s="3">
-        <v>61908</v>
-      </c>
-      <c r="F12" s="4" t="s">
-        <v>15</v>
+        <v>28443</v>
+      </c>
+      <c r="E12" s="6">
+        <v>65737</v>
+      </c>
+      <c r="F12" s="7" t="s">
+        <v>18</v>
       </c>
       <c r="G12" s="2"/>
       <c r="H12" s="2"/>
-      <c r="I12" s="3"/>
+      <c r="I12" s="6"/>
       <c r="J12" s="5"/>
     </row>
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="1"/>
       <c r="B13" s="1" t="s">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="C13" s="2">
-        <v>50675</v>
+        <v>12739</v>
       </c>
       <c r="D13" s="2">
-        <v>22735</v>
+        <v>36270</v>
       </c>
       <c r="E13" s="3">
-        <v>27940</v>
+        <v>-23531</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="G13" s="2"/>
       <c r="H13" s="2"/>
-      <c r="I13" s="3"/>
+      <c r="I13" s="6"/>
       <c r="J13" s="5"/>
     </row>
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="1" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>18</v>
+        <v>3</v>
       </c>
       <c r="C14" s="2">
-        <v>63533</v>
+        <v>84487</v>
       </c>
       <c r="D14" s="2">
-        <v>9623</v>
-      </c>
-      <c r="E14" s="3">
-        <v>53910</v>
-      </c>
-      <c r="F14" s="4" t="s">
-        <v>19</v>
+        <v>48160</v>
+      </c>
+      <c r="E14" s="6">
+        <v>36327</v>
+      </c>
+      <c r="F14" s="7" t="s">
+        <v>21</v>
       </c>
       <c r="G14" s="2">
-        <v>100260</v>
+        <v>180610</v>
       </c>
       <c r="H14" s="2">
-        <v>92780</v>
-      </c>
-      <c r="I14" s="3">
-        <v>7480</v>
+        <v>97882</v>
+      </c>
+      <c r="I14" s="6">
+        <v>82728</v>
       </c>
       <c r="J14" s="8">
-        <v>-75.07</v>
+        <v>3.7900000000000014</v>
       </c>
     </row>
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="1"/>
       <c r="B15" s="1" t="s">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="C15" s="2">
-        <v>25834</v>
+        <v>12674</v>
       </c>
       <c r="D15" s="2">
-        <v>47717</v>
-      </c>
-      <c r="E15" s="6">
-        <v>-21883</v>
-      </c>
-      <c r="F15" s="7" t="s">
-        <v>20</v>
+        <v>25710</v>
+      </c>
+      <c r="E15" s="3">
+        <v>-13036</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>23</v>
       </c>
       <c r="G15" s="2"/>
       <c r="H15" s="2"/>
-      <c r="I15" s="3"/>
+      <c r="I15" s="6"/>
       <c r="J15" s="8"/>
     </row>
     <row r="16" ht="30" customHeight="1">
@@ -697,52 +700,52 @@
         <v>1</v>
       </c>
       <c r="C16" s="2">
-        <v>10893</v>
+        <v>83449</v>
       </c>
       <c r="D16" s="2">
-        <v>35440</v>
+        <v>24012</v>
       </c>
       <c r="E16" s="6">
-        <v>-24547</v>
+        <v>59437</v>
       </c>
       <c r="F16" s="7" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="G16" s="2"/>
       <c r="H16" s="2"/>
-      <c r="I16" s="3"/>
+      <c r="I16" s="6"/>
       <c r="J16" s="8"/>
     </row>
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="1" t="s">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="C17" s="2">
-        <v>16716</v>
+        <v>45948</v>
       </c>
       <c r="D17" s="2">
-        <v>33276</v>
+        <v>23644</v>
       </c>
       <c r="E17" s="6">
-        <v>-16560</v>
+        <v>22304</v>
       </c>
       <c r="F17" s="7" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="G17" s="2">
-        <v>173285</v>
+        <v>123403</v>
       </c>
       <c r="H17" s="2">
-        <v>92420</v>
-      </c>
-      <c r="I17" s="3">
-        <v>80865</v>
-      </c>
-      <c r="J17" s="5">
-        <v>8.520000000000001</v>
+        <v>58829</v>
+      </c>
+      <c r="I17" s="6">
+        <v>64574</v>
+      </c>
+      <c r="J17" s="8">
+        <v>44.89000000000001</v>
       </c>
     </row>
     <row r="18" ht="30" customHeight="1">
@@ -751,249 +754,249 @@
         <v>1</v>
       </c>
       <c r="C18" s="2">
-        <v>75519</v>
+        <v>66049</v>
       </c>
       <c r="D18" s="2">
-        <v>26559</v>
-      </c>
-      <c r="E18" s="3">
-        <v>48960</v>
-      </c>
-      <c r="F18" s="4" t="s">
-        <v>23</v>
+        <v>26830</v>
+      </c>
+      <c r="E18" s="6">
+        <v>39219</v>
+      </c>
+      <c r="F18" s="7" t="s">
+        <v>26</v>
       </c>
       <c r="G18" s="2"/>
       <c r="H18" s="2"/>
-      <c r="I18" s="3"/>
-      <c r="J18" s="5"/>
+      <c r="I18" s="6"/>
+      <c r="J18" s="8"/>
     </row>
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="1"/>
       <c r="B19" s="1" t="s">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="C19" s="2">
-        <v>81050</v>
+        <v>11406</v>
       </c>
       <c r="D19" s="2">
-        <v>32585</v>
-      </c>
-      <c r="E19" s="3">
-        <v>48465</v>
-      </c>
-      <c r="F19" s="4" t="s">
-        <v>24</v>
+        <v>8355</v>
+      </c>
+      <c r="E19" s="6">
+        <v>3051</v>
+      </c>
+      <c r="F19" s="7" t="s">
+        <v>27</v>
       </c>
       <c r="G19" s="2"/>
       <c r="H19" s="2"/>
-      <c r="I19" s="3"/>
-      <c r="J19" s="5"/>
+      <c r="I19" s="6"/>
+      <c r="J19" s="8"/>
     </row>
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="1" t="s">
-        <v>25</v>
+        <v>11</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C20" s="2">
-        <v>72400</v>
+        <v>19838</v>
       </c>
       <c r="D20" s="2">
-        <v>17525</v>
+        <v>48063</v>
       </c>
       <c r="E20" s="3">
-        <v>54875</v>
+        <v>-28225</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="G20" s="2">
-        <v>190025</v>
+        <v>102821</v>
       </c>
       <c r="H20" s="2">
-        <v>83570</v>
-      </c>
-      <c r="I20" s="3">
-        <v>106455</v>
+        <v>101083</v>
+      </c>
+      <c r="I20" s="6">
+        <v>1738</v>
       </c>
       <c r="J20" s="5">
-        <v>32.09</v>
+        <v>-23.793333333333333</v>
       </c>
     </row>
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="1"/>
       <c r="B21" s="1" t="s">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="C21" s="2">
-        <v>28523</v>
+        <v>43435</v>
       </c>
       <c r="D21" s="2">
-        <v>44216</v>
+        <v>21950</v>
       </c>
       <c r="E21" s="6">
-        <v>-15693</v>
+        <v>21485</v>
       </c>
       <c r="F21" s="7" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="G21" s="2"/>
       <c r="H21" s="2"/>
-      <c r="I21" s="3"/>
+      <c r="I21" s="6"/>
       <c r="J21" s="5"/>
     </row>
     <row r="22" ht="30" customHeight="1">
       <c r="A22" s="1"/>
       <c r="B22" s="1" t="s">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="C22" s="2">
-        <v>89102</v>
+        <v>39548</v>
       </c>
       <c r="D22" s="2">
-        <v>21829</v>
-      </c>
-      <c r="E22" s="3">
-        <v>67273</v>
-      </c>
-      <c r="F22" s="4" t="s">
-        <v>28</v>
+        <v>31070</v>
+      </c>
+      <c r="E22" s="6">
+        <v>8478</v>
+      </c>
+      <c r="F22" s="7" t="s">
+        <v>30</v>
       </c>
       <c r="G22" s="2"/>
       <c r="H22" s="2"/>
-      <c r="I22" s="3"/>
+      <c r="I22" s="6"/>
       <c r="J22" s="5"/>
     </row>
     <row r="23" ht="30" customHeight="1">
       <c r="A23" s="1" t="s">
-        <v>29</v>
+        <v>11</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="C23" s="2">
-        <v>53249</v>
+        <v>79556</v>
       </c>
       <c r="D23" s="2">
-        <v>9820</v>
-      </c>
-      <c r="E23" s="3">
-        <v>43429</v>
-      </c>
-      <c r="F23" s="4" t="s">
-        <v>30</v>
+        <v>15356</v>
+      </c>
+      <c r="E23" s="6">
+        <v>64200</v>
+      </c>
+      <c r="F23" s="7" t="s">
+        <v>31</v>
       </c>
       <c r="G23" s="2">
-        <v>235161</v>
+        <v>192111</v>
       </c>
       <c r="H23" s="2">
-        <v>49550</v>
-      </c>
-      <c r="I23" s="3">
-        <v>185611</v>
-      </c>
-      <c r="J23" s="5">
-        <v>79.03333333333335</v>
+        <v>44754</v>
+      </c>
+      <c r="I23" s="6">
+        <v>147357</v>
+      </c>
+      <c r="J23" s="8">
+        <v>77.36666666666667</v>
       </c>
     </row>
     <row r="24" ht="30" customHeight="1">
       <c r="A24" s="1"/>
       <c r="B24" s="1" t="s">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="C24" s="2">
-        <v>94602</v>
+        <v>30154</v>
       </c>
       <c r="D24" s="2">
-        <v>11899</v>
-      </c>
-      <c r="E24" s="3">
-        <v>82703</v>
-      </c>
-      <c r="F24" s="4" t="s">
-        <v>31</v>
+        <v>6149</v>
+      </c>
+      <c r="E24" s="6">
+        <v>24005</v>
+      </c>
+      <c r="F24" s="7" t="s">
+        <v>32</v>
       </c>
       <c r="G24" s="2"/>
       <c r="H24" s="2"/>
-      <c r="I24" s="3"/>
-      <c r="J24" s="5"/>
+      <c r="I24" s="6"/>
+      <c r="J24" s="8"/>
     </row>
     <row r="25" ht="30" customHeight="1">
       <c r="A25" s="1"/>
       <c r="B25" s="1" t="s">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="C25" s="2">
-        <v>87310</v>
+        <v>82401</v>
       </c>
       <c r="D25" s="2">
-        <v>27831</v>
-      </c>
-      <c r="E25" s="3">
-        <v>59479</v>
-      </c>
-      <c r="F25" s="4" t="s">
-        <v>32</v>
+        <v>23249</v>
+      </c>
+      <c r="E25" s="6">
+        <v>59152</v>
+      </c>
+      <c r="F25" s="7" t="s">
+        <v>33</v>
       </c>
       <c r="G25" s="2"/>
       <c r="H25" s="2"/>
-      <c r="I25" s="3"/>
-      <c r="J25" s="5"/>
+      <c r="I25" s="6"/>
+      <c r="J25" s="8"/>
     </row>
     <row r="26" ht="30" customHeight="1">
       <c r="A26" s="1" t="s">
-        <v>0</v>
+        <v>34</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>33</v>
+        <v>1</v>
       </c>
       <c r="C26" s="2">
-        <v>26292</v>
+        <v>60262</v>
       </c>
       <c r="D26" s="2">
-        <v>16206</v>
-      </c>
-      <c r="E26" s="3">
-        <v>10086</v>
-      </c>
-      <c r="F26" s="4" t="s">
-        <v>34</v>
+        <v>30877</v>
+      </c>
+      <c r="E26" s="6">
+        <v>29385</v>
+      </c>
+      <c r="F26" s="7" t="s">
+        <v>35</v>
       </c>
       <c r="G26" s="2">
-        <v>140616</v>
+        <v>161268</v>
       </c>
       <c r="H26" s="2">
-        <v>57174</v>
-      </c>
-      <c r="I26" s="3">
-        <v>83442</v>
-      </c>
-      <c r="J26" s="5">
-        <v>57.71333333333333</v>
+        <v>86335</v>
+      </c>
+      <c r="I26" s="6">
+        <v>74933</v>
+      </c>
+      <c r="J26" s="8">
+        <v>45.723333333333336</v>
       </c>
     </row>
     <row r="27" ht="30" customHeight="1">
       <c r="A27" s="1"/>
       <c r="B27" s="1" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="C27" s="2">
-        <v>69157</v>
+        <v>47463</v>
       </c>
       <c r="D27" s="2">
-        <v>33170</v>
-      </c>
-      <c r="E27" s="3">
-        <v>35987</v>
-      </c>
-      <c r="F27" s="4" t="s">
-        <v>35</v>
+        <v>33505</v>
+      </c>
+      <c r="E27" s="6">
+        <v>13958</v>
+      </c>
+      <c r="F27" s="7" t="s">
+        <v>36</v>
       </c>
       <c r="G27" s="2"/>
       <c r="H27" s="2"/>
-      <c r="I27" s="3"/>
-      <c r="J27" s="5"/>
+      <c r="I27" s="6"/>
+      <c r="J27" s="8"/>
     </row>
     <row r="28" ht="30" customHeight="1">
       <c r="A28" s="1"/>
@@ -1001,110 +1004,110 @@
         <v>1</v>
       </c>
       <c r="C28" s="2">
-        <v>45167</v>
+        <v>53543</v>
       </c>
       <c r="D28" s="2">
-        <v>7798</v>
-      </c>
-      <c r="E28" s="3">
-        <v>37369</v>
-      </c>
-      <c r="F28" s="4" t="s">
-        <v>36</v>
+        <v>21953</v>
+      </c>
+      <c r="E28" s="6">
+        <v>31590</v>
+      </c>
+      <c r="F28" s="7" t="s">
+        <v>37</v>
       </c>
       <c r="G28" s="2"/>
       <c r="H28" s="2"/>
-      <c r="I28" s="3"/>
-      <c r="J28" s="5"/>
+      <c r="I28" s="6"/>
+      <c r="J28" s="8"/>
     </row>
     <row r="29" ht="30" customHeight="1">
       <c r="A29" s="1" t="s">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="C29" s="2">
-        <v>10786</v>
+        <v>41904</v>
       </c>
       <c r="D29" s="2">
-        <v>34900</v>
+        <v>22183</v>
       </c>
       <c r="E29" s="6">
-        <v>-24114</v>
+        <v>19721</v>
       </c>
       <c r="F29" s="7" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="G29" s="2">
-        <v>112706</v>
+        <v>153243</v>
       </c>
       <c r="H29" s="2">
-        <v>60191</v>
-      </c>
-      <c r="I29" s="3">
-        <v>52515</v>
+        <v>60519</v>
+      </c>
+      <c r="I29" s="6">
+        <v>92724</v>
       </c>
       <c r="J29" s="8">
-        <v>-50.43666666666667</v>
+        <v>59.97666666666667</v>
       </c>
     </row>
     <row r="30" ht="30" customHeight="1">
       <c r="A30" s="1"/>
       <c r="B30" s="1" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="C30" s="2">
-        <v>87954</v>
+        <v>24392</v>
       </c>
       <c r="D30" s="2">
-        <v>8857</v>
-      </c>
-      <c r="E30" s="3">
-        <v>79097</v>
-      </c>
-      <c r="F30" s="4" t="s">
-        <v>38</v>
+        <v>7811</v>
+      </c>
+      <c r="E30" s="6">
+        <v>16581</v>
+      </c>
+      <c r="F30" s="7" t="s">
+        <v>39</v>
       </c>
       <c r="G30" s="2"/>
       <c r="H30" s="2"/>
-      <c r="I30" s="3"/>
+      <c r="I30" s="6"/>
       <c r="J30" s="8"/>
     </row>
     <row r="31" ht="30" customHeight="1">
       <c r="A31" s="1"/>
       <c r="B31" s="1" t="s">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="C31" s="2">
-        <v>13966</v>
+        <v>86947</v>
       </c>
       <c r="D31" s="2">
-        <v>16434</v>
+        <v>30525</v>
       </c>
       <c r="E31" s="6">
-        <v>-2468</v>
+        <v>56422</v>
       </c>
       <c r="F31" s="7" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="G31" s="2"/>
       <c r="H31" s="2"/>
-      <c r="I31" s="3"/>
+      <c r="I31" s="6"/>
       <c r="J31" s="8"/>
     </row>
     <row r="32" ht="30" customHeight="1">
       <c r="G32" s="10">
-        <v>1577412</v>
+        <v>1483385</v>
       </c>
       <c r="H32" s="10">
-        <v>747185</v>
+        <v>742927</v>
       </c>
       <c r="I32" s="11">
-        <v>830227</v>
+        <v>740458</v>
       </c>
       <c r="J32" s="12">
-        <v>16.305000000000003</v>
+        <v>27.241666666666667</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs(roadmap): outline report-focused Excel features unlocked by the OOXML writer
Agent-Logs-Url: https://github.com/ChronicStone/typed-xlsx/sessions/e967a859-56f7-4cc7-a3bf-1d7ec66a0493

Co-authored-by: ChronicStone <55083156+ChronicStone@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/packages/typed-xlsx/examples/financial-report-stream.xlsx
+++ b/packages/typed-xlsx/examples/financial-report-stream.xlsx
@@ -10,127 +10,127 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="41">
   <si>
+    <t>2023-11</t>
+  </si>
+  <si>
+    <t>Customer Support</t>
+  </si>
+  <si>
+    <t>1.02%</t>
+  </si>
+  <si>
+    <t>6.33%</t>
+  </si>
+  <si>
+    <t>R&amp;D</t>
+  </si>
+  <si>
+    <t>56.67%</t>
+  </si>
+  <si>
+    <t>2023-05</t>
+  </si>
+  <si>
+    <t>Human Resources</t>
+  </si>
+  <si>
+    <t>28.93%</t>
+  </si>
+  <si>
+    <t>Marketing</t>
+  </si>
+  <si>
+    <t>72.37%</t>
+  </si>
+  <si>
+    <t>64.15%</t>
+  </si>
+  <si>
+    <t>Sales</t>
+  </si>
+  <si>
+    <t>-62.32%</t>
+  </si>
+  <si>
+    <t>69.74%</t>
+  </si>
+  <si>
+    <t>-38.9%</t>
+  </si>
+  <si>
+    <t>2023-03</t>
+  </si>
+  <si>
+    <t>62.54%</t>
+  </si>
+  <si>
+    <t>-73.03%</t>
+  </si>
+  <si>
+    <t>-76.82%</t>
+  </si>
+  <si>
+    <t>2023-04</t>
+  </si>
+  <si>
+    <t>86.64%</t>
+  </si>
+  <si>
+    <t>4.7%</t>
+  </si>
+  <si>
+    <t>82.24%</t>
+  </si>
+  <si>
+    <t>2023-08</t>
+  </si>
+  <si>
+    <t>46.4%</t>
+  </si>
+  <si>
+    <t>56.69%</t>
+  </si>
+  <si>
+    <t>-48.47%</t>
+  </si>
+  <si>
+    <t>27.08%</t>
+  </si>
+  <si>
+    <t>56.53%</t>
+  </si>
+  <si>
+    <t>54.21%</t>
+  </si>
+  <si>
     <t>2023-02</t>
   </si>
   <si>
-    <t>Marketing</t>
-  </si>
-  <si>
-    <t>-87.07%</t>
-  </si>
-  <si>
-    <t>Sales</t>
-  </si>
-  <si>
-    <t>-54.41%</t>
-  </si>
-  <si>
-    <t>Customer Support</t>
-  </si>
-  <si>
-    <t>41.25%</t>
-  </si>
-  <si>
-    <t>2023-12</t>
-  </si>
-  <si>
-    <t>54.67%</t>
-  </si>
-  <si>
-    <t>57.8%</t>
-  </si>
-  <si>
-    <t>86.51%</t>
-  </si>
-  <si>
-    <t>2023-06</t>
-  </si>
-  <si>
-    <t>92.22%</t>
-  </si>
-  <si>
-    <t>-50.82%</t>
-  </si>
-  <si>
-    <t>78.61%</t>
-  </si>
-  <si>
-    <t>2023-01</t>
-  </si>
-  <si>
-    <t>R&amp;D</t>
-  </si>
-  <si>
-    <t>89.55%</t>
-  </si>
-  <si>
-    <t>69.8%</t>
-  </si>
-  <si>
-    <t>-184.72%</t>
-  </si>
-  <si>
-    <t>2023-03</t>
-  </si>
-  <si>
-    <t>43%</t>
-  </si>
-  <si>
-    <t>Human Resources</t>
-  </si>
-  <si>
-    <t>-102.86%</t>
-  </si>
-  <si>
-    <t>71.23%</t>
-  </si>
-  <si>
-    <t>48.54%</t>
-  </si>
-  <si>
-    <t>59.38%</t>
-  </si>
-  <si>
-    <t>26.75%</t>
-  </si>
-  <si>
-    <t>-142.28%</t>
-  </si>
-  <si>
-    <t>49.46%</t>
-  </si>
-  <si>
-    <t>21.44%</t>
-  </si>
-  <si>
-    <t>80.7%</t>
-  </si>
-  <si>
-    <t>79.61%</t>
-  </si>
-  <si>
-    <t>71.79%</t>
-  </si>
-  <si>
-    <t>2023-10</t>
-  </si>
-  <si>
-    <t>48.76%</t>
-  </si>
-  <si>
-    <t>29.41%</t>
-  </si>
-  <si>
-    <t>59%</t>
-  </si>
-  <si>
-    <t>47.06%</t>
-  </si>
-  <si>
-    <t>67.98%</t>
-  </si>
-  <si>
-    <t>64.89%</t>
+    <t>41.72%</t>
+  </si>
+  <si>
+    <t>92.05%</t>
+  </si>
+  <si>
+    <t>57.29%</t>
+  </si>
+  <si>
+    <t>72.65%</t>
+  </si>
+  <si>
+    <t>-84.22%</t>
+  </si>
+  <si>
+    <t>6.42%</t>
+  </si>
+  <si>
+    <t>52.18%</t>
+  </si>
+  <si>
+    <t>-101.93%</t>
+  </si>
+  <si>
+    <t>48.79%</t>
   </si>
 </sst>
 </file>
@@ -147,10 +147,10 @@
       <name val="Calibri"/>
     </font>
     <font>
-      <color rgb="FFFF0000"/>
+      <color rgb="FF007500"/>
     </font>
     <font>
-      <color rgb="FF007500"/>
+      <color rgb="FFFF0000"/>
     </font>
     <font>
       <b/>
@@ -344,46 +344,46 @@
         <v>1</v>
       </c>
       <c r="C2" s="2">
-        <v>26542</v>
+        <v>20336</v>
       </c>
       <c r="D2" s="2">
-        <v>49653</v>
+        <v>20129</v>
       </c>
       <c r="E2" s="3">
-        <v>-23111</v>
+        <v>207</v>
       </c>
       <c r="F2" s="4" t="s">
         <v>2</v>
       </c>
       <c r="G2" s="2">
-        <v>110255</v>
+        <v>118814</v>
       </c>
       <c r="H2" s="2">
-        <v>125998</v>
+        <v>88305</v>
       </c>
       <c r="I2" s="3">
-        <v>-15743</v>
+        <v>30509</v>
       </c>
       <c r="J2" s="5">
-        <v>-33.41</v>
+        <v>21.34</v>
       </c>
     </row>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="1"/>
       <c r="B3" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" s="2">
+        <v>50671</v>
+      </c>
+      <c r="D3" s="2">
+        <v>47462</v>
+      </c>
+      <c r="E3" s="3">
+        <v>3209</v>
+      </c>
+      <c r="F3" s="4" t="s">
         <v>3</v>
-      </c>
-      <c r="C3" s="2">
-        <v>28398</v>
-      </c>
-      <c r="D3" s="2">
-        <v>43848</v>
-      </c>
-      <c r="E3" s="3">
-        <v>-15450</v>
-      </c>
-      <c r="F3" s="4" t="s">
-        <v>4</v>
       </c>
       <c r="G3" s="2"/>
       <c r="H3" s="2"/>
@@ -393,19 +393,19 @@
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="1"/>
       <c r="B4" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C4" s="2">
+        <v>47807</v>
+      </c>
+      <c r="D4" s="2">
+        <v>20714</v>
+      </c>
+      <c r="E4" s="3">
+        <v>27093</v>
+      </c>
+      <c r="F4" s="4" t="s">
         <v>5</v>
-      </c>
-      <c r="C4" s="2">
-        <v>55315</v>
-      </c>
-      <c r="D4" s="2">
-        <v>32497</v>
-      </c>
-      <c r="E4" s="6">
-        <v>22818</v>
-      </c>
-      <c r="F4" s="7" t="s">
-        <v>6</v>
       </c>
       <c r="G4" s="2"/>
       <c r="H4" s="2"/>
@@ -414,361 +414,361 @@
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="1" t="s">
-        <v>5</v>
-      </c>
       <c r="C5" s="2">
-        <v>80795</v>
+        <v>57053</v>
       </c>
       <c r="D5" s="2">
-        <v>36626</v>
-      </c>
-      <c r="E5" s="6">
-        <v>44169</v>
-      </c>
-      <c r="F5" s="7" t="s">
+        <v>40547</v>
+      </c>
+      <c r="E5" s="3">
+        <v>16506</v>
+      </c>
+      <c r="F5" s="4" t="s">
         <v>8</v>
       </c>
       <c r="G5" s="2">
-        <v>156044</v>
+        <v>193493</v>
       </c>
       <c r="H5" s="2">
-        <v>55124</v>
-      </c>
-      <c r="I5" s="6">
-        <v>100920</v>
-      </c>
-      <c r="J5" s="8">
-        <v>66.32666666666667</v>
+        <v>82129</v>
+      </c>
+      <c r="I5" s="3">
+        <v>111364</v>
+      </c>
+      <c r="J5" s="5">
+        <v>55.150000000000006</v>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="1"/>
       <c r="B6" s="1" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="C6" s="2">
-        <v>29071</v>
+        <v>89221</v>
       </c>
       <c r="D6" s="2">
-        <v>12267</v>
-      </c>
-      <c r="E6" s="6">
-        <v>16804</v>
-      </c>
-      <c r="F6" s="7" t="s">
-        <v>9</v>
+        <v>24653</v>
+      </c>
+      <c r="E6" s="3">
+        <v>64568</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="G6" s="2"/>
       <c r="H6" s="2"/>
-      <c r="I6" s="6"/>
-      <c r="J6" s="8"/>
+      <c r="I6" s="3"/>
+      <c r="J6" s="5"/>
     </row>
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="1"/>
       <c r="B7" s="1" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="C7" s="2">
-        <v>46178</v>
+        <v>47219</v>
       </c>
       <c r="D7" s="2">
-        <v>6231</v>
-      </c>
-      <c r="E7" s="6">
-        <v>39947</v>
-      </c>
-      <c r="F7" s="7" t="s">
-        <v>10</v>
+        <v>16929</v>
+      </c>
+      <c r="E7" s="3">
+        <v>30290</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>11</v>
       </c>
       <c r="G7" s="2"/>
       <c r="H7" s="2"/>
-      <c r="I7" s="6"/>
-      <c r="J7" s="8"/>
+      <c r="I7" s="3"/>
+      <c r="J7" s="5"/>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="1" t="s">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="C8" s="2">
-        <v>77643</v>
+        <v>27693</v>
       </c>
       <c r="D8" s="2">
-        <v>6038</v>
+        <v>44952</v>
       </c>
       <c r="E8" s="6">
-        <v>71605</v>
+        <v>-17259</v>
       </c>
       <c r="F8" s="7" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G8" s="2">
-        <v>120670</v>
+        <v>121865</v>
       </c>
       <c r="H8" s="2">
-        <v>39747</v>
-      </c>
-      <c r="I8" s="6">
-        <v>80923</v>
+        <v>100475</v>
+      </c>
+      <c r="I8" s="3">
+        <v>21390</v>
       </c>
       <c r="J8" s="8">
-        <v>40.00333333333333</v>
+        <v>-10.493333333333334</v>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="1"/>
       <c r="B9" s="1" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="C9" s="2">
-        <v>18933</v>
+        <v>69292</v>
       </c>
       <c r="D9" s="2">
-        <v>28555</v>
+        <v>20965</v>
       </c>
       <c r="E9" s="3">
-        <v>-9622</v>
+        <v>48327</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G9" s="2"/>
       <c r="H9" s="2"/>
-      <c r="I9" s="6"/>
+      <c r="I9" s="3"/>
       <c r="J9" s="8"/>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="1"/>
       <c r="B10" s="1" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C10" s="2">
-        <v>24094</v>
+        <v>24880</v>
       </c>
       <c r="D10" s="2">
-        <v>5154</v>
+        <v>34558</v>
       </c>
       <c r="E10" s="6">
-        <v>18940</v>
+        <v>-9678</v>
       </c>
       <c r="F10" s="7" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G10" s="2"/>
       <c r="H10" s="2"/>
-      <c r="I10" s="6"/>
+      <c r="I10" s="3"/>
       <c r="J10" s="8"/>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="C11" s="2">
-        <v>76041</v>
+        <v>55793</v>
       </c>
       <c r="D11" s="2">
-        <v>7943</v>
-      </c>
-      <c r="E11" s="6">
-        <v>68098</v>
-      </c>
-      <c r="F11" s="7" t="s">
+        <v>20901</v>
+      </c>
+      <c r="E11" s="3">
+        <v>34892</v>
+      </c>
+      <c r="F11" s="4" t="s">
         <v>17</v>
       </c>
       <c r="G11" s="2">
-        <v>182960</v>
+        <v>84437</v>
       </c>
       <c r="H11" s="2">
-        <v>72656</v>
-      </c>
-      <c r="I11" s="6">
-        <v>110304</v>
-      </c>
-      <c r="J11" s="5">
-        <v>-8.456666666666669</v>
+        <v>71068</v>
+      </c>
+      <c r="I11" s="3">
+        <v>13369</v>
+      </c>
+      <c r="J11" s="8">
+        <v>-29.103333333333335</v>
       </c>
     </row>
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="1"/>
       <c r="B12" s="1" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="C12" s="2">
-        <v>94180</v>
+        <v>12694</v>
       </c>
       <c r="D12" s="2">
-        <v>28443</v>
+        <v>21965</v>
       </c>
       <c r="E12" s="6">
-        <v>65737</v>
+        <v>-9271</v>
       </c>
       <c r="F12" s="7" t="s">
         <v>18</v>
       </c>
       <c r="G12" s="2"/>
       <c r="H12" s="2"/>
-      <c r="I12" s="6"/>
-      <c r="J12" s="5"/>
+      <c r="I12" s="3"/>
+      <c r="J12" s="8"/>
     </row>
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="1"/>
       <c r="B13" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C13" s="2">
-        <v>12739</v>
+        <v>15950</v>
       </c>
       <c r="D13" s="2">
-        <v>36270</v>
-      </c>
-      <c r="E13" s="3">
-        <v>-23531</v>
-      </c>
-      <c r="F13" s="4" t="s">
+        <v>28202</v>
+      </c>
+      <c r="E13" s="6">
+        <v>-12252</v>
+      </c>
+      <c r="F13" s="7" t="s">
         <v>19</v>
       </c>
       <c r="G13" s="2"/>
       <c r="H13" s="2"/>
-      <c r="I13" s="6"/>
-      <c r="J13" s="5"/>
+      <c r="I13" s="3"/>
+      <c r="J13" s="8"/>
     </row>
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="1" t="s">
         <v>20</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C14" s="2">
-        <v>84487</v>
+        <v>46631</v>
       </c>
       <c r="D14" s="2">
-        <v>48160</v>
-      </c>
-      <c r="E14" s="6">
-        <v>36327</v>
-      </c>
-      <c r="F14" s="7" t="s">
+        <v>6231</v>
+      </c>
+      <c r="E14" s="3">
+        <v>40400</v>
+      </c>
+      <c r="F14" s="4" t="s">
         <v>21</v>
       </c>
       <c r="G14" s="2">
-        <v>180610</v>
+        <v>142750</v>
       </c>
       <c r="H14" s="2">
-        <v>97882</v>
-      </c>
-      <c r="I14" s="6">
-        <v>82728</v>
-      </c>
-      <c r="J14" s="8">
-        <v>3.7900000000000014</v>
+        <v>49857</v>
+      </c>
+      <c r="I14" s="3">
+        <v>92893</v>
+      </c>
+      <c r="J14" s="5">
+        <v>57.85999999999999</v>
       </c>
     </row>
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="1"/>
       <c r="B15" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C15" s="2">
+        <v>34243</v>
+      </c>
+      <c r="D15" s="2">
+        <v>32635</v>
+      </c>
+      <c r="E15" s="3">
+        <v>1608</v>
+      </c>
+      <c r="F15" s="4" t="s">
         <v>22</v>
-      </c>
-      <c r="C15" s="2">
-        <v>12674</v>
-      </c>
-      <c r="D15" s="2">
-        <v>25710</v>
-      </c>
-      <c r="E15" s="3">
-        <v>-13036</v>
-      </c>
-      <c r="F15" s="4" t="s">
-        <v>23</v>
       </c>
       <c r="G15" s="2"/>
       <c r="H15" s="2"/>
-      <c r="I15" s="6"/>
-      <c r="J15" s="8"/>
+      <c r="I15" s="3"/>
+      <c r="J15" s="5"/>
     </row>
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="1"/>
       <c r="B16" s="1" t="s">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="C16" s="2">
-        <v>83449</v>
+        <v>61876</v>
       </c>
       <c r="D16" s="2">
-        <v>24012</v>
-      </c>
-      <c r="E16" s="6">
-        <v>59437</v>
-      </c>
-      <c r="F16" s="7" t="s">
-        <v>24</v>
+        <v>10991</v>
+      </c>
+      <c r="E16" s="3">
+        <v>50885</v>
+      </c>
+      <c r="F16" s="4" t="s">
+        <v>23</v>
       </c>
       <c r="G16" s="2"/>
       <c r="H16" s="2"/>
-      <c r="I16" s="6"/>
-      <c r="J16" s="8"/>
+      <c r="I16" s="3"/>
+      <c r="J16" s="5"/>
     </row>
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="1" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="C17" s="2">
-        <v>45948</v>
+        <v>33537</v>
       </c>
       <c r="D17" s="2">
-        <v>23644</v>
-      </c>
-      <c r="E17" s="6">
-        <v>22304</v>
-      </c>
-      <c r="F17" s="7" t="s">
+        <v>17976</v>
+      </c>
+      <c r="E17" s="3">
+        <v>15561</v>
+      </c>
+      <c r="F17" s="4" t="s">
         <v>25</v>
       </c>
       <c r="G17" s="2">
-        <v>123403</v>
+        <v>145994</v>
       </c>
       <c r="H17" s="2">
-        <v>58829</v>
-      </c>
-      <c r="I17" s="6">
-        <v>64574</v>
-      </c>
-      <c r="J17" s="8">
-        <v>44.89000000000001</v>
+        <v>86431</v>
+      </c>
+      <c r="I17" s="3">
+        <v>59563</v>
+      </c>
+      <c r="J17" s="5">
+        <v>18.206666666666667</v>
       </c>
     </row>
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="1"/>
       <c r="B18" s="1" t="s">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C18" s="2">
-        <v>66049</v>
+        <v>93676</v>
       </c>
       <c r="D18" s="2">
-        <v>26830</v>
-      </c>
-      <c r="E18" s="6">
-        <v>39219</v>
-      </c>
-      <c r="F18" s="7" t="s">
+        <v>40571</v>
+      </c>
+      <c r="E18" s="3">
+        <v>53105</v>
+      </c>
+      <c r="F18" s="4" t="s">
         <v>26</v>
       </c>
       <c r="G18" s="2"/>
       <c r="H18" s="2"/>
-      <c r="I18" s="6"/>
-      <c r="J18" s="8"/>
+      <c r="I18" s="3"/>
+      <c r="J18" s="5"/>
     </row>
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="1"/>
@@ -776,74 +776,74 @@
         <v>1</v>
       </c>
       <c r="C19" s="2">
-        <v>11406</v>
+        <v>18781</v>
       </c>
       <c r="D19" s="2">
-        <v>8355</v>
+        <v>27884</v>
       </c>
       <c r="E19" s="6">
-        <v>3051</v>
+        <v>-9103</v>
       </c>
       <c r="F19" s="7" t="s">
         <v>27</v>
       </c>
       <c r="G19" s="2"/>
       <c r="H19" s="2"/>
-      <c r="I19" s="6"/>
-      <c r="J19" s="8"/>
+      <c r="I19" s="3"/>
+      <c r="J19" s="5"/>
     </row>
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="1" t="s">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="C20" s="2">
-        <v>19838</v>
+        <v>33514</v>
       </c>
       <c r="D20" s="2">
-        <v>48063</v>
+        <v>24438</v>
       </c>
       <c r="E20" s="3">
-        <v>-28225</v>
+        <v>9076</v>
       </c>
       <c r="F20" s="4" t="s">
         <v>28</v>
       </c>
       <c r="G20" s="2">
-        <v>102821</v>
+        <v>97453</v>
       </c>
       <c r="H20" s="2">
-        <v>101083</v>
-      </c>
-      <c r="I20" s="6">
-        <v>1738</v>
+        <v>52865</v>
+      </c>
+      <c r="I20" s="3">
+        <v>44588</v>
       </c>
       <c r="J20" s="5">
-        <v>-23.793333333333333</v>
+        <v>45.94</v>
       </c>
     </row>
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="1"/>
       <c r="B21" s="1" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="C21" s="2">
-        <v>43435</v>
+        <v>36682</v>
       </c>
       <c r="D21" s="2">
-        <v>21950</v>
-      </c>
-      <c r="E21" s="6">
-        <v>21485</v>
-      </c>
-      <c r="F21" s="7" t="s">
+        <v>15946</v>
+      </c>
+      <c r="E21" s="3">
+        <v>20736</v>
+      </c>
+      <c r="F21" s="4" t="s">
         <v>29</v>
       </c>
       <c r="G21" s="2"/>
       <c r="H21" s="2"/>
-      <c r="I21" s="6"/>
+      <c r="I21" s="3"/>
       <c r="J21" s="5"/>
     </row>
     <row r="22" ht="30" customHeight="1">
@@ -852,262 +852,262 @@
         <v>1</v>
       </c>
       <c r="C22" s="2">
-        <v>39548</v>
+        <v>27257</v>
       </c>
       <c r="D22" s="2">
-        <v>31070</v>
-      </c>
-      <c r="E22" s="6">
-        <v>8478</v>
-      </c>
-      <c r="F22" s="7" t="s">
+        <v>12481</v>
+      </c>
+      <c r="E22" s="3">
+        <v>14776</v>
+      </c>
+      <c r="F22" s="4" t="s">
         <v>30</v>
       </c>
       <c r="G22" s="2"/>
       <c r="H22" s="2"/>
-      <c r="I22" s="6"/>
+      <c r="I22" s="3"/>
       <c r="J22" s="5"/>
     </row>
     <row r="23" ht="30" customHeight="1">
       <c r="A23" s="1" t="s">
-        <v>11</v>
+        <v>31</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="C23" s="2">
-        <v>79556</v>
+        <v>54349</v>
       </c>
       <c r="D23" s="2">
-        <v>15356</v>
-      </c>
-      <c r="E23" s="6">
-        <v>64200</v>
-      </c>
-      <c r="F23" s="7" t="s">
-        <v>31</v>
+        <v>31676</v>
+      </c>
+      <c r="E23" s="3">
+        <v>22673</v>
+      </c>
+      <c r="F23" s="4" t="s">
+        <v>32</v>
       </c>
       <c r="G23" s="2">
-        <v>192111</v>
+        <v>239410</v>
       </c>
       <c r="H23" s="2">
-        <v>44754</v>
-      </c>
-      <c r="I23" s="6">
-        <v>147357</v>
-      </c>
-      <c r="J23" s="8">
-        <v>77.36666666666667</v>
+        <v>78973</v>
+      </c>
+      <c r="I23" s="3">
+        <v>160437</v>
+      </c>
+      <c r="J23" s="5">
+        <v>63.68666666666666</v>
       </c>
     </row>
     <row r="24" ht="30" customHeight="1">
       <c r="A24" s="1"/>
       <c r="B24" s="1" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C24" s="2">
-        <v>30154</v>
+        <v>91318</v>
       </c>
       <c r="D24" s="2">
-        <v>6149</v>
-      </c>
-      <c r="E24" s="6">
-        <v>24005</v>
-      </c>
-      <c r="F24" s="7" t="s">
-        <v>32</v>
+        <v>7261</v>
+      </c>
+      <c r="E24" s="3">
+        <v>84057</v>
+      </c>
+      <c r="F24" s="4" t="s">
+        <v>33</v>
       </c>
       <c r="G24" s="2"/>
       <c r="H24" s="2"/>
-      <c r="I24" s="6"/>
-      <c r="J24" s="8"/>
+      <c r="I24" s="3"/>
+      <c r="J24" s="5"/>
     </row>
     <row r="25" ht="30" customHeight="1">
       <c r="A25" s="1"/>
       <c r="B25" s="1" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C25" s="2">
-        <v>82401</v>
+        <v>93743</v>
       </c>
       <c r="D25" s="2">
-        <v>23249</v>
-      </c>
-      <c r="E25" s="6">
-        <v>59152</v>
-      </c>
-      <c r="F25" s="7" t="s">
-        <v>33</v>
+        <v>40036</v>
+      </c>
+      <c r="E25" s="3">
+        <v>53707</v>
+      </c>
+      <c r="F25" s="4" t="s">
+        <v>34</v>
       </c>
       <c r="G25" s="2"/>
       <c r="H25" s="2"/>
-      <c r="I25" s="6"/>
-      <c r="J25" s="8"/>
+      <c r="I25" s="3"/>
+      <c r="J25" s="5"/>
     </row>
     <row r="26" ht="30" customHeight="1">
       <c r="A26" s="1" t="s">
-        <v>34</v>
+        <v>0</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="C26" s="2">
-        <v>60262</v>
+        <v>89985</v>
       </c>
       <c r="D26" s="2">
-        <v>30877</v>
-      </c>
-      <c r="E26" s="6">
-        <v>29385</v>
-      </c>
-      <c r="F26" s="7" t="s">
+        <v>24613</v>
+      </c>
+      <c r="E26" s="3">
+        <v>65372</v>
+      </c>
+      <c r="F26" s="4" t="s">
         <v>35</v>
       </c>
       <c r="G26" s="2">
-        <v>161268</v>
+        <v>150796</v>
       </c>
       <c r="H26" s="2">
-        <v>86335</v>
-      </c>
-      <c r="I26" s="6">
-        <v>74933</v>
+        <v>100621</v>
+      </c>
+      <c r="I26" s="3">
+        <v>50175</v>
       </c>
       <c r="J26" s="8">
-        <v>45.723333333333336</v>
+        <v>-1.7166666666666643</v>
       </c>
     </row>
     <row r="27" ht="30" customHeight="1">
       <c r="A27" s="1"/>
       <c r="B27" s="1" t="s">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="C27" s="2">
-        <v>47463</v>
+        <v>21074</v>
       </c>
       <c r="D27" s="2">
-        <v>33505</v>
+        <v>38822</v>
       </c>
       <c r="E27" s="6">
-        <v>13958</v>
+        <v>-17748</v>
       </c>
       <c r="F27" s="7" t="s">
         <v>36</v>
       </c>
       <c r="G27" s="2"/>
       <c r="H27" s="2"/>
-      <c r="I27" s="6"/>
+      <c r="I27" s="3"/>
       <c r="J27" s="8"/>
     </row>
     <row r="28" ht="30" customHeight="1">
       <c r="A28" s="1"/>
       <c r="B28" s="1" t="s">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="C28" s="2">
-        <v>53543</v>
+        <v>39737</v>
       </c>
       <c r="D28" s="2">
-        <v>21953</v>
-      </c>
-      <c r="E28" s="6">
-        <v>31590</v>
-      </c>
-      <c r="F28" s="7" t="s">
+        <v>37186</v>
+      </c>
+      <c r="E28" s="3">
+        <v>2551</v>
+      </c>
+      <c r="F28" s="4" t="s">
         <v>37</v>
       </c>
       <c r="G28" s="2"/>
       <c r="H28" s="2"/>
-      <c r="I28" s="6"/>
+      <c r="I28" s="3"/>
       <c r="J28" s="8"/>
     </row>
     <row r="29" ht="30" customHeight="1">
       <c r="A29" s="1" t="s">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C29" s="2">
-        <v>41904</v>
+        <v>96072</v>
       </c>
       <c r="D29" s="2">
-        <v>22183</v>
-      </c>
-      <c r="E29" s="6">
-        <v>19721</v>
-      </c>
-      <c r="F29" s="7" t="s">
+        <v>45945</v>
+      </c>
+      <c r="E29" s="3">
+        <v>50127</v>
+      </c>
+      <c r="F29" s="4" t="s">
         <v>38</v>
       </c>
       <c r="G29" s="2">
-        <v>153243</v>
+        <v>172403</v>
       </c>
       <c r="H29" s="2">
-        <v>60519</v>
-      </c>
-      <c r="I29" s="6">
-        <v>92724</v>
+        <v>122288</v>
+      </c>
+      <c r="I29" s="3">
+        <v>50115</v>
       </c>
       <c r="J29" s="8">
-        <v>59.97666666666667</v>
+        <v>-0.32000000000000267</v>
       </c>
     </row>
     <row r="30" ht="30" customHeight="1">
       <c r="A30" s="1"/>
       <c r="B30" s="1" t="s">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="C30" s="2">
-        <v>24392</v>
+        <v>24717</v>
       </c>
       <c r="D30" s="2">
-        <v>7811</v>
+        <v>49910</v>
       </c>
       <c r="E30" s="6">
-        <v>16581</v>
+        <v>-25193</v>
       </c>
       <c r="F30" s="7" t="s">
         <v>39</v>
       </c>
       <c r="G30" s="2"/>
       <c r="H30" s="2"/>
-      <c r="I30" s="6"/>
+      <c r="I30" s="3"/>
       <c r="J30" s="8"/>
     </row>
     <row r="31" ht="30" customHeight="1">
       <c r="A31" s="1"/>
       <c r="B31" s="1" t="s">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C31" s="2">
-        <v>86947</v>
+        <v>51614</v>
       </c>
       <c r="D31" s="2">
-        <v>30525</v>
-      </c>
-      <c r="E31" s="6">
-        <v>56422</v>
-      </c>
-      <c r="F31" s="7" t="s">
+        <v>26433</v>
+      </c>
+      <c r="E31" s="3">
+        <v>25181</v>
+      </c>
+      <c r="F31" s="4" t="s">
         <v>40</v>
       </c>
       <c r="G31" s="2"/>
       <c r="H31" s="2"/>
-      <c r="I31" s="6"/>
+      <c r="I31" s="3"/>
       <c r="J31" s="8"/>
     </row>
     <row r="32" ht="30" customHeight="1">
       <c r="G32" s="10">
-        <v>1483385</v>
+        <v>1467415</v>
       </c>
       <c r="H32" s="10">
-        <v>742927</v>
+        <v>833012</v>
       </c>
       <c r="I32" s="11">
-        <v>740458</v>
+        <v>634403</v>
       </c>
       <c r="J32" s="12">
-        <v>27.241666666666667</v>
+        <v>22.055</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(core): add conditional styling support
</commit_message>
<xml_diff>
--- a/packages/typed-xlsx/examples/financial-report-stream.xlsx
+++ b/packages/typed-xlsx/examples/financial-report-stream.xlsx
@@ -8,132 +8,123 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="42">
-  <si>
-    <t>2023-10</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="39">
+  <si>
+    <t>2023-08</t>
+  </si>
+  <si>
+    <t>Human Resources</t>
+  </si>
+  <si>
+    <t>-144.93%</t>
+  </si>
+  <si>
+    <t>58.86%</t>
+  </si>
+  <si>
+    <t>Sales</t>
+  </si>
+  <si>
+    <t>73.41%</t>
+  </si>
+  <si>
+    <t>2023-05</t>
+  </si>
+  <si>
+    <t>82.01%</t>
   </si>
   <si>
     <t>R&amp;D</t>
   </si>
   <si>
-    <t>-80.78%</t>
-  </si>
-  <si>
-    <t>Human Resources</t>
-  </si>
-  <si>
-    <t>84.91%</t>
-  </si>
-  <si>
-    <t>89.14%</t>
+    <t>37.44%</t>
+  </si>
+  <si>
+    <t>42.04%</t>
+  </si>
+  <si>
+    <t>2023-12</t>
+  </si>
+  <si>
+    <t>63.98%</t>
+  </si>
+  <si>
+    <t>62.72%</t>
+  </si>
+  <si>
+    <t>35.8%</t>
   </si>
   <si>
     <t>2023-11</t>
   </si>
   <si>
+    <t>56.12%</t>
+  </si>
+  <si>
+    <t>77.5%</t>
+  </si>
+  <si>
+    <t>29.01%</t>
+  </si>
+  <si>
     <t>Marketing</t>
   </si>
   <si>
-    <t>75.1%</t>
+    <t>57.92%</t>
   </si>
   <si>
     <t>Customer Support</t>
   </si>
   <si>
-    <t>72.58%</t>
-  </si>
-  <si>
-    <t>Sales</t>
-  </si>
-  <si>
-    <t>67.93%</t>
-  </si>
-  <si>
-    <t>2023-01</t>
-  </si>
-  <si>
-    <t>58.17%</t>
-  </si>
-  <si>
-    <t>69.74%</t>
-  </si>
-  <si>
-    <t>52.15%</t>
-  </si>
-  <si>
-    <t>2023-04</t>
-  </si>
-  <si>
-    <t>52.96%</t>
-  </si>
-  <si>
-    <t>79.43%</t>
-  </si>
-  <si>
-    <t>17.78%</t>
-  </si>
-  <si>
-    <t>72.85%</t>
-  </si>
-  <si>
-    <t>41.41%</t>
-  </si>
-  <si>
-    <t>41.42%</t>
-  </si>
-  <si>
-    <t>27.45%</t>
-  </si>
-  <si>
-    <t>73.41%</t>
-  </si>
-  <si>
-    <t>55.01%</t>
-  </si>
-  <si>
-    <t>2023-09</t>
-  </si>
-  <si>
-    <t>84.4%</t>
-  </si>
-  <si>
-    <t>8.8%</t>
-  </si>
-  <si>
-    <t>55.49%</t>
-  </si>
-  <si>
-    <t>2023-03</t>
-  </si>
-  <si>
-    <t>77.86%</t>
-  </si>
-  <si>
-    <t>89.36%</t>
-  </si>
-  <si>
-    <t>75.8%</t>
-  </si>
-  <si>
-    <t>2023-08</t>
-  </si>
-  <si>
-    <t>42.84%</t>
-  </si>
-  <si>
-    <t>-21.86%</t>
-  </si>
-  <si>
-    <t>22.18%</t>
-  </si>
-  <si>
-    <t>41.94%</t>
-  </si>
-  <si>
-    <t>70.15%</t>
-  </si>
-  <si>
-    <t>-19.51%</t>
+    <t>51.25%</t>
+  </si>
+  <si>
+    <t>42.05%</t>
+  </si>
+  <si>
+    <t>-98.06%</t>
+  </si>
+  <si>
+    <t>51.65%</t>
+  </si>
+  <si>
+    <t>54.34%</t>
+  </si>
+  <si>
+    <t>29.91%</t>
+  </si>
+  <si>
+    <t>21.63%</t>
+  </si>
+  <si>
+    <t>63.61%</t>
+  </si>
+  <si>
+    <t>36.03%</t>
+  </si>
+  <si>
+    <t>76.16%</t>
+  </si>
+  <si>
+    <t>41.93%</t>
+  </si>
+  <si>
+    <t>-78.54%</t>
+  </si>
+  <si>
+    <t>60.38%</t>
+  </si>
+  <si>
+    <t>44.41%</t>
+  </si>
+  <si>
+    <t>34.41%</t>
+  </si>
+  <si>
+    <t>33.8%</t>
+  </si>
+  <si>
+    <t>53.1%</t>
   </si>
 </sst>
 </file>
@@ -225,7 +216,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -242,10 +233,13 @@
     <xf numFmtId="164" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="165" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="165" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -267,6 +261,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
 </styleSheet>
 </file>
 
@@ -288,52 +283,52 @@
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
-      <c r="A1" t="inlineStr" s="10">
+      <c r="A1" t="inlineStr" s="11">
         <is>
           <t>Month</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr" s="10">
+      <c r="B1" t="inlineStr" s="11">
         <is>
           <t>Department</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr" s="10">
+      <c r="C1" t="inlineStr" s="11">
         <is>
           <t>Revenue</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr" s="10">
+      <c r="D1" t="inlineStr" s="11">
         <is>
           <t>Expenses</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr" s="10">
+      <c r="E1" t="inlineStr" s="11">
         <is>
           <t>Profit</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr" s="10">
+      <c r="F1" t="inlineStr" s="11">
         <is>
           <t>Profit Margin</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr" s="10">
+      <c r="G1" t="inlineStr" s="11">
         <is>
           <t>Total Revenue</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr" s="10">
+      <c r="H1" t="inlineStr" s="11">
         <is>
           <t>Total Expenses</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr" s="10">
+      <c r="I1" t="inlineStr" s="11">
         <is>
           <t>Total Profit</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr" s="10">
+      <c r="J1" t="inlineStr" s="11">
         <is>
           <t>Average Profit Margin</t>
         </is>
@@ -347,46 +342,46 @@
         <v>1</v>
       </c>
       <c r="C2" s="2">
-        <v>17077</v>
+        <v>15022</v>
       </c>
       <c r="D2" s="2">
-        <v>30872</v>
+        <v>36794</v>
       </c>
       <c r="E2" s="3">
-        <v>-13795</v>
+        <v>-21772</v>
       </c>
       <c r="F2" s="4" t="s">
         <v>2</v>
       </c>
       <c r="G2" s="2">
-        <v>169367</v>
+        <v>152958</v>
       </c>
       <c r="H2" s="2">
-        <v>49960</v>
+        <v>82638</v>
       </c>
       <c r="I2" s="5">
-        <v>119407</v>
+        <v>70320</v>
       </c>
       <c r="J2" s="6">
-        <v>31.09</v>
+        <v>-4.220000000000003</v>
       </c>
     </row>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="1"/>
       <c r="B3" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" s="2">
+        <v>62995</v>
+      </c>
+      <c r="D3" s="2">
+        <v>25917</v>
+      </c>
+      <c r="E3" s="5">
+        <v>37078</v>
+      </c>
+      <c r="F3" s="7" t="s">
         <v>3</v>
-      </c>
-      <c r="C3" s="2">
-        <v>60252</v>
-      </c>
-      <c r="D3" s="2">
-        <v>9090</v>
-      </c>
-      <c r="E3" s="5">
-        <v>51162</v>
-      </c>
-      <c r="F3" s="7" t="s">
-        <v>4</v>
       </c>
       <c r="G3" s="2"/>
       <c r="H3" s="2"/>
@@ -396,16 +391,16 @@
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="1"/>
       <c r="B4" s="1" t="s">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C4" s="2">
-        <v>92038</v>
+        <v>74941</v>
       </c>
       <c r="D4" s="2">
-        <v>9998</v>
+        <v>19927</v>
       </c>
       <c r="E4" s="5">
-        <v>82040</v>
+        <v>55014</v>
       </c>
       <c r="F4" s="7" t="s">
         <v>5</v>
@@ -420,274 +415,274 @@
         <v>6</v>
       </c>
       <c r="B5" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C5" s="2">
+        <v>90406</v>
+      </c>
+      <c r="D5" s="2">
+        <v>16263</v>
+      </c>
+      <c r="E5" s="5">
+        <v>74143</v>
+      </c>
+      <c r="F5" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="C5" s="2">
-        <v>57672</v>
-      </c>
-      <c r="D5" s="2">
-        <v>14358</v>
-      </c>
-      <c r="E5" s="5">
-        <v>43314</v>
-      </c>
-      <c r="F5" s="7" t="s">
-        <v>8</v>
-      </c>
       <c r="G5" s="2">
-        <v>220599</v>
+        <v>185078</v>
       </c>
       <c r="H5" s="2">
-        <v>62999</v>
+        <v>72753</v>
       </c>
       <c r="I5" s="5">
-        <v>157600</v>
-      </c>
-      <c r="J5" s="6">
-        <v>71.87</v>
+        <v>112325</v>
+      </c>
+      <c r="J5" s="8">
+        <v>53.830000000000005</v>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="1"/>
       <c r="B6" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C6" s="2">
+        <v>35191</v>
+      </c>
+      <c r="D6" s="2">
+        <v>22017</v>
+      </c>
+      <c r="E6" s="5">
+        <v>13174</v>
+      </c>
+      <c r="F6" s="7" t="s">
         <v>9</v>
-      </c>
-      <c r="C6" s="2">
-        <v>77546</v>
-      </c>
-      <c r="D6" s="2">
-        <v>21260</v>
-      </c>
-      <c r="E6" s="5">
-        <v>56286</v>
-      </c>
-      <c r="F6" s="7" t="s">
-        <v>10</v>
       </c>
       <c r="G6" s="2"/>
       <c r="H6" s="2"/>
       <c r="I6" s="5"/>
-      <c r="J6" s="6"/>
+      <c r="J6" s="8"/>
     </row>
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="1"/>
       <c r="B7" s="1" t="s">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="C7" s="2">
-        <v>85381</v>
+        <v>59481</v>
       </c>
       <c r="D7" s="2">
-        <v>27381</v>
+        <v>34473</v>
       </c>
       <c r="E7" s="5">
-        <v>58000</v>
+        <v>25008</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="G7" s="2"/>
       <c r="H7" s="2"/>
       <c r="I7" s="5"/>
-      <c r="J7" s="6"/>
+      <c r="J7" s="8"/>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="1" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="C8" s="2">
-        <v>33936</v>
+        <v>51065</v>
       </c>
       <c r="D8" s="2">
-        <v>14196</v>
+        <v>18392</v>
       </c>
       <c r="E8" s="5">
-        <v>19740</v>
+        <v>32673</v>
       </c>
       <c r="F8" s="7" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="G8" s="2">
-        <v>224963</v>
+        <v>207488</v>
       </c>
       <c r="H8" s="2">
-        <v>88165</v>
+        <v>92839</v>
       </c>
       <c r="I8" s="5">
-        <v>136798</v>
-      </c>
-      <c r="J8" s="6">
-        <v>60.02</v>
+        <v>114649</v>
+      </c>
+      <c r="J8" s="8">
+        <v>54.166666666666664</v>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="1"/>
       <c r="B9" s="1" t="s">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="C9" s="2">
-        <v>99143</v>
+        <v>96507</v>
       </c>
       <c r="D9" s="2">
-        <v>30000</v>
+        <v>35978</v>
       </c>
       <c r="E9" s="5">
-        <v>69143</v>
+        <v>60529</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="G9" s="2"/>
       <c r="H9" s="2"/>
       <c r="I9" s="5"/>
-      <c r="J9" s="6"/>
+      <c r="J9" s="8"/>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="1"/>
       <c r="B10" s="1" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C10" s="2">
-        <v>91884</v>
+        <v>59916</v>
       </c>
       <c r="D10" s="2">
-        <v>43969</v>
+        <v>38469</v>
       </c>
       <c r="E10" s="5">
-        <v>47915</v>
+        <v>21447</v>
       </c>
       <c r="F10" s="7" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="G10" s="2"/>
       <c r="H10" s="2"/>
       <c r="I10" s="5"/>
-      <c r="J10" s="6"/>
+      <c r="J10" s="8"/>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="1" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C11" s="2">
-        <v>49457</v>
+        <v>85681</v>
       </c>
       <c r="D11" s="2">
-        <v>23264</v>
+        <v>37597</v>
       </c>
       <c r="E11" s="5">
-        <v>26193</v>
+        <v>48084</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="G11" s="2">
-        <v>188600</v>
+        <v>197528</v>
       </c>
       <c r="H11" s="2">
-        <v>78282</v>
+        <v>89533</v>
       </c>
       <c r="I11" s="5">
-        <v>110318</v>
-      </c>
-      <c r="J11" s="6">
-        <v>50.05666666666667</v>
+        <v>107995</v>
+      </c>
+      <c r="J11" s="8">
+        <v>54.21</v>
       </c>
     </row>
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="1"/>
       <c r="B12" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C12" s="2">
-        <v>96326</v>
+        <v>56633</v>
       </c>
       <c r="D12" s="2">
-        <v>19814</v>
+        <v>12742</v>
       </c>
       <c r="E12" s="5">
-        <v>76512</v>
+        <v>43891</v>
       </c>
       <c r="F12" s="7" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="G12" s="2"/>
       <c r="H12" s="2"/>
       <c r="I12" s="5"/>
-      <c r="J12" s="6"/>
+      <c r="J12" s="8"/>
     </row>
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="1"/>
       <c r="B13" s="1" t="s">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="C13" s="2">
-        <v>42817</v>
+        <v>55214</v>
       </c>
       <c r="D13" s="2">
-        <v>35204</v>
+        <v>39194</v>
       </c>
       <c r="E13" s="5">
-        <v>7613</v>
+        <v>16020</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="G13" s="2"/>
       <c r="H13" s="2"/>
       <c r="I13" s="5"/>
-      <c r="J13" s="6"/>
+      <c r="J13" s="8"/>
     </row>
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="C14" s="2">
-        <v>94547</v>
+        <v>77549</v>
       </c>
       <c r="D14" s="2">
-        <v>25674</v>
+        <v>32633</v>
       </c>
       <c r="E14" s="5">
-        <v>68873</v>
+        <v>44916</v>
       </c>
       <c r="F14" s="7" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G14" s="2">
-        <v>189153</v>
+        <v>193595</v>
       </c>
       <c r="H14" s="2">
-        <v>81097</v>
+        <v>94900</v>
       </c>
       <c r="I14" s="5">
-        <v>108056</v>
-      </c>
-      <c r="J14" s="6">
-        <v>51.89333333333334</v>
+        <v>98695</v>
+      </c>
+      <c r="J14" s="8">
+        <v>50.406666666666666</v>
       </c>
     </row>
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="1"/>
       <c r="B15" s="1" t="s">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="C15" s="2">
-        <v>47581</v>
+        <v>54155</v>
       </c>
       <c r="D15" s="2">
-        <v>27876</v>
+        <v>26402</v>
       </c>
       <c r="E15" s="5">
-        <v>19705</v>
+        <v>27753</v>
       </c>
       <c r="F15" s="7" t="s">
         <v>22</v>
@@ -695,21 +690,21 @@
       <c r="G15" s="2"/>
       <c r="H15" s="2"/>
       <c r="I15" s="5"/>
-      <c r="J15" s="6"/>
+      <c r="J15" s="8"/>
     </row>
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="1"/>
       <c r="B16" s="1" t="s">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="C16" s="2">
-        <v>47025</v>
+        <v>61891</v>
       </c>
       <c r="D16" s="2">
-        <v>27547</v>
+        <v>35865</v>
       </c>
       <c r="E16" s="5">
-        <v>19478</v>
+        <v>26026</v>
       </c>
       <c r="F16" s="7" t="s">
         <v>23</v>
@@ -717,53 +712,53 @@
       <c r="G16" s="2"/>
       <c r="H16" s="2"/>
       <c r="I16" s="5"/>
-      <c r="J16" s="6"/>
+      <c r="J16" s="8"/>
     </row>
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="1" t="s">
-        <v>17</v>
+        <v>6</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="C17" s="2">
-        <v>67738</v>
+        <v>13229</v>
       </c>
       <c r="D17" s="2">
-        <v>49142</v>
-      </c>
-      <c r="E17" s="5">
-        <v>18596</v>
-      </c>
-      <c r="F17" s="7" t="s">
+        <v>26202</v>
+      </c>
+      <c r="E17" s="3">
+        <v>-12973</v>
+      </c>
+      <c r="F17" s="4" t="s">
         <v>24</v>
       </c>
       <c r="G17" s="2">
-        <v>161540</v>
+        <v>113342</v>
       </c>
       <c r="H17" s="2">
-        <v>80634</v>
+        <v>74242</v>
       </c>
       <c r="I17" s="5">
-        <v>80906</v>
-      </c>
-      <c r="J17" s="6">
-        <v>51.95666666666667</v>
+        <v>39100</v>
+      </c>
+      <c r="J17" s="8">
+        <v>2.643333333333333</v>
       </c>
     </row>
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="1"/>
       <c r="B18" s="1" t="s">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="C18" s="2">
-        <v>58213</v>
+        <v>86656</v>
       </c>
       <c r="D18" s="2">
-        <v>15481</v>
+        <v>41895</v>
       </c>
       <c r="E18" s="5">
-        <v>42732</v>
+        <v>44761</v>
       </c>
       <c r="F18" s="7" t="s">
         <v>25</v>
@@ -771,21 +766,21 @@
       <c r="G18" s="2"/>
       <c r="H18" s="2"/>
       <c r="I18" s="5"/>
-      <c r="J18" s="6"/>
+      <c r="J18" s="8"/>
     </row>
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="1"/>
       <c r="B19" s="1" t="s">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="C19" s="2">
-        <v>35589</v>
+        <v>13457</v>
       </c>
       <c r="D19" s="2">
-        <v>16011</v>
+        <v>6145</v>
       </c>
       <c r="E19" s="5">
-        <v>19578</v>
+        <v>7312</v>
       </c>
       <c r="F19" s="7" t="s">
         <v>26</v>
@@ -793,324 +788,324 @@
       <c r="G19" s="2"/>
       <c r="H19" s="2"/>
       <c r="I19" s="5"/>
-      <c r="J19" s="6"/>
+      <c r="J19" s="8"/>
     </row>
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C20" s="2">
+        <v>56463</v>
+      </c>
+      <c r="D20" s="2">
+        <v>39576</v>
+      </c>
+      <c r="E20" s="5">
+        <v>16887</v>
+      </c>
+      <c r="F20" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="B20" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C20" s="2">
-        <v>46347</v>
-      </c>
-      <c r="D20" s="2">
-        <v>7228</v>
-      </c>
-      <c r="E20" s="5">
-        <v>39119</v>
-      </c>
-      <c r="F20" s="7" t="s">
-        <v>28</v>
-      </c>
       <c r="G20" s="2">
-        <v>179596</v>
+        <v>193279</v>
       </c>
       <c r="H20" s="2">
-        <v>85916</v>
+        <v>107783</v>
       </c>
       <c r="I20" s="5">
-        <v>93680</v>
-      </c>
-      <c r="J20" s="6">
-        <v>49.56333333333333</v>
+        <v>85496</v>
+      </c>
+      <c r="J20" s="8">
+        <v>38.38333333333333</v>
       </c>
     </row>
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="1"/>
       <c r="B21" s="1" t="s">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C21" s="2">
-        <v>41501</v>
+        <v>43871</v>
       </c>
       <c r="D21" s="2">
-        <v>37849</v>
+        <v>34380</v>
       </c>
       <c r="E21" s="5">
-        <v>3652</v>
+        <v>9491</v>
       </c>
       <c r="F21" s="7" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="G21" s="2"/>
       <c r="H21" s="2"/>
       <c r="I21" s="5"/>
-      <c r="J21" s="6"/>
+      <c r="J21" s="8"/>
     </row>
     <row r="22" ht="30" customHeight="1">
       <c r="A22" s="1"/>
       <c r="B22" s="1" t="s">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="C22" s="2">
-        <v>91748</v>
+        <v>92945</v>
       </c>
       <c r="D22" s="2">
-        <v>40839</v>
+        <v>33827</v>
       </c>
       <c r="E22" s="5">
-        <v>50909</v>
+        <v>59118</v>
       </c>
       <c r="F22" s="7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="G22" s="2"/>
       <c r="H22" s="2"/>
       <c r="I22" s="5"/>
-      <c r="J22" s="6"/>
+      <c r="J22" s="8"/>
     </row>
     <row r="23" ht="30" customHeight="1">
       <c r="A23" s="1" t="s">
-        <v>31</v>
+        <v>15</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="C23" s="2">
-        <v>91267</v>
+        <v>75236</v>
       </c>
       <c r="D23" s="2">
-        <v>20210</v>
+        <v>48132</v>
       </c>
       <c r="E23" s="5">
-        <v>71057</v>
+        <v>27104</v>
       </c>
       <c r="F23" s="7" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="G23" s="2">
-        <v>247959</v>
+        <v>219138</v>
       </c>
       <c r="H23" s="2">
-        <v>46183</v>
+        <v>98135</v>
       </c>
       <c r="I23" s="5">
-        <v>201776</v>
-      </c>
-      <c r="J23" s="6">
-        <v>81.00666666666666</v>
+        <v>121003</v>
+      </c>
+      <c r="J23" s="8">
+        <v>51.373333333333335</v>
       </c>
     </row>
     <row r="24" ht="30" customHeight="1">
       <c r="A24" s="1"/>
       <c r="B24" s="1" t="s">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C24" s="2">
-        <v>88091</v>
+        <v>98047</v>
       </c>
       <c r="D24" s="2">
-        <v>9374</v>
+        <v>23375</v>
       </c>
       <c r="E24" s="5">
-        <v>78717</v>
+        <v>74672</v>
       </c>
       <c r="F24" s="7" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="G24" s="2"/>
       <c r="H24" s="2"/>
       <c r="I24" s="5"/>
-      <c r="J24" s="6"/>
+      <c r="J24" s="8"/>
     </row>
     <row r="25" ht="30" customHeight="1">
       <c r="A25" s="1"/>
       <c r="B25" s="1" t="s">
-        <v>3</v>
+        <v>21</v>
       </c>
       <c r="C25" s="2">
-        <v>68601</v>
+        <v>45855</v>
       </c>
       <c r="D25" s="2">
-        <v>16599</v>
+        <v>26628</v>
       </c>
       <c r="E25" s="5">
-        <v>52002</v>
+        <v>19227</v>
       </c>
       <c r="F25" s="7" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="G25" s="2"/>
       <c r="H25" s="2"/>
       <c r="I25" s="5"/>
-      <c r="J25" s="6"/>
+      <c r="J25" s="8"/>
     </row>
     <row r="26" ht="30" customHeight="1">
       <c r="A26" s="1" t="s">
-        <v>35</v>
+        <v>6</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="C26" s="2">
-        <v>22160</v>
+        <v>27114</v>
       </c>
       <c r="D26" s="2">
-        <v>12666</v>
-      </c>
-      <c r="E26" s="5">
-        <v>9494</v>
-      </c>
-      <c r="F26" s="7" t="s">
-        <v>36</v>
+        <v>48410</v>
+      </c>
+      <c r="E26" s="3">
+        <v>-21296</v>
+      </c>
+      <c r="F26" s="4" t="s">
+        <v>33</v>
       </c>
       <c r="G26" s="2">
-        <v>69395</v>
+        <v>180909</v>
       </c>
       <c r="H26" s="2">
-        <v>54759</v>
+        <v>118999</v>
       </c>
       <c r="I26" s="5">
-        <v>14636</v>
-      </c>
-      <c r="J26" s="6">
-        <v>14.386666666666668</v>
+        <v>61910</v>
+      </c>
+      <c r="J26" s="8">
+        <v>8.749999999999998</v>
       </c>
     </row>
     <row r="27" ht="30" customHeight="1">
       <c r="A27" s="1"/>
       <c r="B27" s="1" t="s">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="C27" s="2">
-        <v>12111</v>
+        <v>93297</v>
       </c>
       <c r="D27" s="2">
-        <v>14758</v>
-      </c>
-      <c r="E27" s="3">
-        <v>-2647</v>
-      </c>
-      <c r="F27" s="4" t="s">
-        <v>37</v>
+        <v>36960</v>
+      </c>
+      <c r="E27" s="5">
+        <v>56337</v>
+      </c>
+      <c r="F27" s="7" t="s">
+        <v>34</v>
       </c>
       <c r="G27" s="2"/>
       <c r="H27" s="2"/>
       <c r="I27" s="5"/>
-      <c r="J27" s="6"/>
+      <c r="J27" s="8"/>
     </row>
     <row r="28" ht="30" customHeight="1">
       <c r="A28" s="1"/>
       <c r="B28" s="1" t="s">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="C28" s="2">
-        <v>35124</v>
+        <v>60498</v>
       </c>
       <c r="D28" s="2">
-        <v>27335</v>
+        <v>33629</v>
       </c>
       <c r="E28" s="5">
-        <v>7789</v>
+        <v>26869</v>
       </c>
       <c r="F28" s="7" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="G28" s="2"/>
       <c r="H28" s="2"/>
       <c r="I28" s="5"/>
-      <c r="J28" s="6"/>
+      <c r="J28" s="8"/>
     </row>
     <row r="29" ht="30" customHeight="1">
       <c r="A29" s="1" t="s">
-        <v>31</v>
+        <v>11</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="C29" s="2">
-        <v>74551</v>
+        <v>69704</v>
       </c>
       <c r="D29" s="2">
-        <v>43284</v>
+        <v>45718</v>
       </c>
       <c r="E29" s="5">
-        <v>31267</v>
+        <v>23986</v>
       </c>
       <c r="F29" s="7" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="G29" s="2">
-        <v>184410</v>
+        <v>151085</v>
       </c>
       <c r="H29" s="2">
-        <v>89606</v>
+        <v>87765</v>
       </c>
       <c r="I29" s="5">
-        <v>94804</v>
-      </c>
-      <c r="J29" s="6">
-        <v>30.86</v>
+        <v>63320</v>
+      </c>
+      <c r="J29" s="8">
+        <v>40.43666666666667</v>
       </c>
     </row>
     <row r="30" ht="30" customHeight="1">
       <c r="A30" s="1"/>
       <c r="B30" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C30" s="2">
-        <v>94767</v>
+        <v>20102</v>
       </c>
       <c r="D30" s="2">
-        <v>28286</v>
+        <v>13308</v>
       </c>
       <c r="E30" s="5">
-        <v>66481</v>
+        <v>6794</v>
       </c>
       <c r="F30" s="7" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="G30" s="2"/>
       <c r="H30" s="2"/>
       <c r="I30" s="5"/>
-      <c r="J30" s="6"/>
+      <c r="J30" s="8"/>
     </row>
     <row r="31" ht="30" customHeight="1">
       <c r="A31" s="1"/>
       <c r="B31" s="1" t="s">
-        <v>3</v>
+        <v>19</v>
       </c>
       <c r="C31" s="2">
-        <v>15092</v>
+        <v>61279</v>
       </c>
       <c r="D31" s="2">
-        <v>18036</v>
-      </c>
-      <c r="E31" s="3">
-        <v>-2944</v>
-      </c>
-      <c r="F31" s="4" t="s">
-        <v>41</v>
+        <v>28739</v>
+      </c>
+      <c r="E31" s="5">
+        <v>32540</v>
+      </c>
+      <c r="F31" s="7" t="s">
+        <v>38</v>
       </c>
       <c r="G31" s="2"/>
       <c r="H31" s="2"/>
       <c r="I31" s="5"/>
-      <c r="J31" s="6"/>
+      <c r="J31" s="8"/>
     </row>
     <row r="32" ht="30" customHeight="1">
-      <c r="G32" s="9">
-        <v>1835582</v>
-      </c>
-      <c r="H32" s="9">
-        <v>717601</v>
-      </c>
-      <c r="I32" s="11">
-        <v>1117981</v>
-      </c>
-      <c r="J32" s="12">
-        <v>49.27033333333333</v>
+      <c r="G32" s="10">
+        <v>1794400</v>
+      </c>
+      <c r="H32" s="10">
+        <v>919587</v>
+      </c>
+      <c r="I32" s="12">
+        <v>874813</v>
+      </c>
+      <c r="J32" s="13">
+        <v>34.998000000000005</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
refactor(core): remove vnext layout
</commit_message>
<xml_diff>
--- a/packages/typed-xlsx/examples/financial-report-stream.xlsx
+++ b/packages/typed-xlsx/examples/financial-report-stream.xlsx
@@ -8,123 +8,135 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="39">
-  <si>
-    <t>2023-08</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="43">
+  <si>
+    <t>2023-12</t>
+  </si>
+  <si>
+    <t>Customer Support</t>
+  </si>
+  <si>
+    <t>-310.19%</t>
+  </si>
+  <si>
+    <t>R&amp;D</t>
+  </si>
+  <si>
+    <t>46.65%</t>
+  </si>
+  <si>
+    <t>Marketing</t>
+  </si>
+  <si>
+    <t>73.2%</t>
+  </si>
+  <si>
+    <t>2023-09</t>
+  </si>
+  <si>
+    <t>70.63%</t>
+  </si>
+  <si>
+    <t>-37.95%</t>
+  </si>
+  <si>
+    <t>50.77%</t>
+  </si>
+  <si>
+    <t>2023-03</t>
+  </si>
+  <si>
+    <t>36.12%</t>
   </si>
   <si>
     <t>Human Resources</t>
   </si>
   <si>
-    <t>-144.93%</t>
-  </si>
-  <si>
-    <t>58.86%</t>
+    <t>89.12%</t>
+  </si>
+  <si>
+    <t>-34.95%</t>
+  </si>
+  <si>
+    <t>2023-11</t>
+  </si>
+  <si>
+    <t>91.28%</t>
+  </si>
+  <si>
+    <t>53.04%</t>
+  </si>
+  <si>
+    <t>14.21%</t>
+  </si>
+  <si>
+    <t>-46.19%</t>
+  </si>
+  <si>
+    <t>70.19%</t>
+  </si>
+  <si>
+    <t>63.49%</t>
+  </si>
+  <si>
+    <t>2023-04</t>
+  </si>
+  <si>
+    <t>17.85%</t>
+  </si>
+  <si>
+    <t>29.76%</t>
+  </si>
+  <si>
+    <t>85.11%</t>
+  </si>
+  <si>
+    <t>2023-02</t>
+  </si>
+  <si>
+    <t>53.94%</t>
+  </si>
+  <si>
+    <t>26.94%</t>
+  </si>
+  <si>
+    <t>8.78%</t>
+  </si>
+  <si>
+    <t>2023-01</t>
   </si>
   <si>
     <t>Sales</t>
   </si>
   <si>
-    <t>73.41%</t>
-  </si>
-  <si>
-    <t>2023-05</t>
-  </si>
-  <si>
-    <t>82.01%</t>
-  </si>
-  <si>
-    <t>R&amp;D</t>
-  </si>
-  <si>
-    <t>37.44%</t>
-  </si>
-  <si>
-    <t>42.04%</t>
-  </si>
-  <si>
-    <t>2023-12</t>
-  </si>
-  <si>
-    <t>63.98%</t>
-  </si>
-  <si>
-    <t>62.72%</t>
-  </si>
-  <si>
-    <t>35.8%</t>
-  </si>
-  <si>
-    <t>2023-11</t>
-  </si>
-  <si>
-    <t>56.12%</t>
-  </si>
-  <si>
-    <t>77.5%</t>
+    <t>64.4%</t>
+  </si>
+  <si>
+    <t>91.31%</t>
+  </si>
+  <si>
+    <t>36.71%</t>
+  </si>
+  <si>
+    <t>2023-07</t>
+  </si>
+  <si>
+    <t>47.75%</t>
+  </si>
+  <si>
+    <t>22.38%</t>
+  </si>
+  <si>
+    <t>88.12%</t>
   </si>
   <si>
     <t>29.01%</t>
   </si>
   <si>
-    <t>Marketing</t>
-  </si>
-  <si>
-    <t>57.92%</t>
-  </si>
-  <si>
-    <t>Customer Support</t>
-  </si>
-  <si>
-    <t>51.25%</t>
-  </si>
-  <si>
-    <t>42.05%</t>
-  </si>
-  <si>
-    <t>-98.06%</t>
-  </si>
-  <si>
-    <t>51.65%</t>
-  </si>
-  <si>
-    <t>54.34%</t>
-  </si>
-  <si>
-    <t>29.91%</t>
-  </si>
-  <si>
-    <t>21.63%</t>
-  </si>
-  <si>
-    <t>63.61%</t>
-  </si>
-  <si>
-    <t>36.03%</t>
-  </si>
-  <si>
-    <t>76.16%</t>
-  </si>
-  <si>
-    <t>41.93%</t>
-  </si>
-  <si>
-    <t>-78.54%</t>
-  </si>
-  <si>
-    <t>60.38%</t>
-  </si>
-  <si>
-    <t>44.41%</t>
-  </si>
-  <si>
-    <t>34.41%</t>
-  </si>
-  <si>
-    <t>33.8%</t>
-  </si>
-  <si>
-    <t>53.1%</t>
+    <t>77.28%</t>
+  </si>
+  <si>
+    <t>92.81%</t>
   </si>
 </sst>
 </file>
@@ -342,46 +354,46 @@
         <v>1</v>
       </c>
       <c r="C2" s="2">
-        <v>15022</v>
+        <v>11020</v>
       </c>
       <c r="D2" s="2">
-        <v>36794</v>
+        <v>45203</v>
       </c>
       <c r="E2" s="3">
-        <v>-21772</v>
+        <v>-34183</v>
       </c>
       <c r="F2" s="4" t="s">
         <v>2</v>
       </c>
       <c r="G2" s="2">
-        <v>152958</v>
+        <v>146693</v>
       </c>
       <c r="H2" s="2">
-        <v>82638</v>
+        <v>93690</v>
       </c>
       <c r="I2" s="5">
-        <v>70320</v>
+        <v>53003</v>
       </c>
       <c r="J2" s="6">
-        <v>-4.220000000000003</v>
+        <v>-63.44666666666668</v>
       </c>
     </row>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="1"/>
       <c r="B3" s="1" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C3" s="2">
-        <v>62995</v>
+        <v>45676</v>
       </c>
       <c r="D3" s="2">
-        <v>25917</v>
+        <v>24369</v>
       </c>
       <c r="E3" s="5">
-        <v>37078</v>
+        <v>21307</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G3" s="2"/>
       <c r="H3" s="2"/>
@@ -391,19 +403,19 @@
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="1"/>
       <c r="B4" s="1" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C4" s="2">
-        <v>74941</v>
+        <v>89997</v>
       </c>
       <c r="D4" s="2">
-        <v>19927</v>
+        <v>24118</v>
       </c>
       <c r="E4" s="5">
-        <v>55014</v>
+        <v>65879</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G4" s="2"/>
       <c r="H4" s="2"/>
@@ -412,51 +424,51 @@
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C5" s="2">
-        <v>90406</v>
+        <v>35786</v>
       </c>
       <c r="D5" s="2">
-        <v>16263</v>
+        <v>10510</v>
       </c>
       <c r="E5" s="5">
-        <v>74143</v>
+        <v>25276</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G5" s="2">
-        <v>185078</v>
+        <v>94558</v>
       </c>
       <c r="H5" s="2">
-        <v>72753</v>
+        <v>56561</v>
       </c>
       <c r="I5" s="5">
-        <v>112325</v>
+        <v>37997</v>
       </c>
       <c r="J5" s="8">
-        <v>53.830000000000005</v>
+        <v>27.816666666666663</v>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="1"/>
       <c r="B6" s="1" t="s">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="C6" s="2">
-        <v>35191</v>
+        <v>19296</v>
       </c>
       <c r="D6" s="2">
-        <v>22017</v>
-      </c>
-      <c r="E6" s="5">
-        <v>13174</v>
-      </c>
-      <c r="F6" s="7" t="s">
+        <v>26618</v>
+      </c>
+      <c r="E6" s="3">
+        <v>-7322</v>
+      </c>
+      <c r="F6" s="4" t="s">
         <v>9</v>
       </c>
       <c r="G6" s="2"/>
@@ -467,16 +479,16 @@
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="1"/>
       <c r="B7" s="1" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C7" s="2">
-        <v>59481</v>
+        <v>39476</v>
       </c>
       <c r="D7" s="2">
-        <v>34473</v>
+        <v>19433</v>
       </c>
       <c r="E7" s="5">
-        <v>25008</v>
+        <v>20043</v>
       </c>
       <c r="F7" s="7" t="s">
         <v>10</v>
@@ -491,49 +503,49 @@
         <v>11</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C8" s="2">
-        <v>51065</v>
+        <v>15519</v>
       </c>
       <c r="D8" s="2">
-        <v>18392</v>
+        <v>9914</v>
       </c>
       <c r="E8" s="5">
-        <v>32673</v>
+        <v>5605</v>
       </c>
       <c r="F8" s="7" t="s">
         <v>12</v>
       </c>
       <c r="G8" s="2">
-        <v>207488</v>
+        <v>121042</v>
       </c>
       <c r="H8" s="2">
-        <v>92839</v>
+        <v>63386</v>
       </c>
       <c r="I8" s="5">
-        <v>114649</v>
+        <v>57656</v>
       </c>
       <c r="J8" s="8">
-        <v>54.166666666666664</v>
+        <v>30.096666666666668</v>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="1"/>
       <c r="B9" s="1" t="s">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="C9" s="2">
-        <v>96507</v>
+        <v>71676</v>
       </c>
       <c r="D9" s="2">
-        <v>35978</v>
+        <v>7797</v>
       </c>
       <c r="E9" s="5">
-        <v>60529</v>
+        <v>63879</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G9" s="2"/>
       <c r="H9" s="2"/>
@@ -543,19 +555,19 @@
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="1"/>
       <c r="B10" s="1" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C10" s="2">
-        <v>59916</v>
+        <v>33847</v>
       </c>
       <c r="D10" s="2">
-        <v>38469</v>
-      </c>
-      <c r="E10" s="5">
-        <v>21447</v>
-      </c>
-      <c r="F10" s="7" t="s">
-        <v>14</v>
+        <v>45675</v>
+      </c>
+      <c r="E10" s="3">
+        <v>-11828</v>
+      </c>
+      <c r="F10" s="4" t="s">
+        <v>15</v>
       </c>
       <c r="G10" s="2"/>
       <c r="H10" s="2"/>
@@ -564,52 +576,52 @@
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C11" s="2">
-        <v>85681</v>
+        <v>83517</v>
       </c>
       <c r="D11" s="2">
-        <v>37597</v>
+        <v>7285</v>
       </c>
       <c r="E11" s="5">
-        <v>48084</v>
+        <v>76232</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G11" s="2">
-        <v>197528</v>
+        <v>218949</v>
       </c>
       <c r="H11" s="2">
-        <v>89533</v>
+        <v>88432</v>
       </c>
       <c r="I11" s="5">
-        <v>107995</v>
+        <v>130517</v>
       </c>
       <c r="J11" s="8">
-        <v>54.21</v>
+        <v>52.843333333333334</v>
       </c>
     </row>
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="1"/>
       <c r="B12" s="1" t="s">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="C12" s="2">
-        <v>56633</v>
+        <v>90250</v>
       </c>
       <c r="D12" s="2">
-        <v>12742</v>
+        <v>42384</v>
       </c>
       <c r="E12" s="5">
-        <v>43891</v>
+        <v>47866</v>
       </c>
       <c r="F12" s="7" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="G12" s="2"/>
       <c r="H12" s="2"/>
@@ -619,19 +631,19 @@
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="1"/>
       <c r="B13" s="1" t="s">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="C13" s="2">
-        <v>55214</v>
+        <v>45182</v>
       </c>
       <c r="D13" s="2">
-        <v>39194</v>
+        <v>38763</v>
       </c>
       <c r="E13" s="5">
-        <v>16020</v>
+        <v>6419</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="G13" s="2"/>
       <c r="H13" s="2"/>
@@ -640,52 +652,52 @@
     </row>
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="1" t="s">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="C14" s="2">
-        <v>77549</v>
+        <v>25010</v>
       </c>
       <c r="D14" s="2">
-        <v>32633</v>
-      </c>
-      <c r="E14" s="5">
-        <v>44916</v>
-      </c>
-      <c r="F14" s="7" t="s">
+        <v>36562</v>
+      </c>
+      <c r="E14" s="3">
+        <v>-11552</v>
+      </c>
+      <c r="F14" s="4" t="s">
         <v>20</v>
       </c>
       <c r="G14" s="2">
-        <v>193595</v>
+        <v>169731</v>
       </c>
       <c r="H14" s="2">
-        <v>94900</v>
+        <v>85448</v>
       </c>
       <c r="I14" s="5">
-        <v>98695</v>
+        <v>84283</v>
       </c>
       <c r="J14" s="8">
-        <v>50.406666666666666</v>
+        <v>29.163333333333338</v>
       </c>
     </row>
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="1"/>
       <c r="B15" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C15" s="2">
+        <v>58889</v>
+      </c>
+      <c r="D15" s="2">
+        <v>17553</v>
+      </c>
+      <c r="E15" s="5">
+        <v>41336</v>
+      </c>
+      <c r="F15" s="7" t="s">
         <v>21</v>
-      </c>
-      <c r="C15" s="2">
-        <v>54155</v>
-      </c>
-      <c r="D15" s="2">
-        <v>26402</v>
-      </c>
-      <c r="E15" s="5">
-        <v>27753</v>
-      </c>
-      <c r="F15" s="7" t="s">
-        <v>22</v>
       </c>
       <c r="G15" s="2"/>
       <c r="H15" s="2"/>
@@ -695,19 +707,19 @@
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="1"/>
       <c r="B16" s="1" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="C16" s="2">
-        <v>61891</v>
+        <v>85832</v>
       </c>
       <c r="D16" s="2">
-        <v>35865</v>
+        <v>31333</v>
       </c>
       <c r="E16" s="5">
-        <v>26026</v>
+        <v>54499</v>
       </c>
       <c r="F16" s="7" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G16" s="2"/>
       <c r="H16" s="2"/>
@@ -716,49 +728,49 @@
     </row>
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="1" t="s">
-        <v>6</v>
+        <v>23</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="C17" s="2">
-        <v>13229</v>
+        <v>59271</v>
       </c>
       <c r="D17" s="2">
-        <v>26202</v>
-      </c>
-      <c r="E17" s="3">
-        <v>-12973</v>
-      </c>
-      <c r="F17" s="4" t="s">
+        <v>48689</v>
+      </c>
+      <c r="E17" s="5">
+        <v>10582</v>
+      </c>
+      <c r="F17" s="7" t="s">
         <v>24</v>
       </c>
       <c r="G17" s="2">
-        <v>113342</v>
+        <v>188391</v>
       </c>
       <c r="H17" s="2">
-        <v>74242</v>
+        <v>100311</v>
       </c>
       <c r="I17" s="5">
-        <v>39100</v>
+        <v>88080</v>
       </c>
       <c r="J17" s="8">
-        <v>2.643333333333333</v>
+        <v>44.24</v>
       </c>
     </row>
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="1"/>
       <c r="B18" s="1" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C18" s="2">
-        <v>86656</v>
+        <v>58526</v>
       </c>
       <c r="D18" s="2">
-        <v>41895</v>
+        <v>41111</v>
       </c>
       <c r="E18" s="5">
-        <v>44761</v>
+        <v>17415</v>
       </c>
       <c r="F18" s="7" t="s">
         <v>25</v>
@@ -771,16 +783,16 @@
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="1"/>
       <c r="B19" s="1" t="s">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="C19" s="2">
-        <v>13457</v>
+        <v>70594</v>
       </c>
       <c r="D19" s="2">
-        <v>6145</v>
+        <v>10511</v>
       </c>
       <c r="E19" s="5">
-        <v>7312</v>
+        <v>60083</v>
       </c>
       <c r="F19" s="7" t="s">
         <v>26</v>
@@ -792,52 +804,52 @@
     </row>
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="1" t="s">
-        <v>6</v>
+        <v>27</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="C20" s="2">
-        <v>56463</v>
+        <v>98904</v>
       </c>
       <c r="D20" s="2">
-        <v>39576</v>
+        <v>45553</v>
       </c>
       <c r="E20" s="5">
-        <v>16887</v>
+        <v>53351</v>
       </c>
       <c r="F20" s="7" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G20" s="2">
-        <v>193279</v>
+        <v>209634</v>
       </c>
       <c r="H20" s="2">
-        <v>107783</v>
+        <v>134807</v>
       </c>
       <c r="I20" s="5">
-        <v>85496</v>
+        <v>74827</v>
       </c>
       <c r="J20" s="8">
-        <v>38.38333333333333</v>
+        <v>29.886666666666667</v>
       </c>
     </row>
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="1"/>
       <c r="B21" s="1" t="s">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="C21" s="2">
-        <v>43871</v>
+        <v>64724</v>
       </c>
       <c r="D21" s="2">
-        <v>34380</v>
+        <v>47288</v>
       </c>
       <c r="E21" s="5">
-        <v>9491</v>
+        <v>17436</v>
       </c>
       <c r="F21" s="7" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G21" s="2"/>
       <c r="H21" s="2"/>
@@ -847,19 +859,19 @@
     <row r="22" ht="30" customHeight="1">
       <c r="A22" s="1"/>
       <c r="B22" s="1" t="s">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="C22" s="2">
-        <v>92945</v>
+        <v>46006</v>
       </c>
       <c r="D22" s="2">
-        <v>33827</v>
+        <v>41966</v>
       </c>
       <c r="E22" s="5">
-        <v>59118</v>
+        <v>4040</v>
       </c>
       <c r="F22" s="7" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="G22" s="2"/>
       <c r="H22" s="2"/>
@@ -868,52 +880,52 @@
     </row>
     <row r="23" ht="30" customHeight="1">
       <c r="A23" s="1" t="s">
-        <v>15</v>
+        <v>31</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>1</v>
+        <v>32</v>
       </c>
       <c r="C23" s="2">
-        <v>75236</v>
+        <v>95945</v>
       </c>
       <c r="D23" s="2">
-        <v>48132</v>
+        <v>34159</v>
       </c>
       <c r="E23" s="5">
-        <v>27104</v>
+        <v>61786</v>
       </c>
       <c r="F23" s="7" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="G23" s="2">
-        <v>219138</v>
+        <v>244928</v>
       </c>
       <c r="H23" s="2">
-        <v>98135</v>
+        <v>81268</v>
       </c>
       <c r="I23" s="5">
-        <v>121003</v>
+        <v>163660</v>
       </c>
       <c r="J23" s="8">
-        <v>51.373333333333335</v>
+        <v>64.14</v>
       </c>
     </row>
     <row r="24" ht="30" customHeight="1">
       <c r="A24" s="1"/>
       <c r="B24" s="1" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C24" s="2">
-        <v>98047</v>
+        <v>86421</v>
       </c>
       <c r="D24" s="2">
-        <v>23375</v>
+        <v>7512</v>
       </c>
       <c r="E24" s="5">
-        <v>74672</v>
+        <v>78909</v>
       </c>
       <c r="F24" s="7" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="G24" s="2"/>
       <c r="H24" s="2"/>
@@ -923,19 +935,19 @@
     <row r="25" ht="30" customHeight="1">
       <c r="A25" s="1"/>
       <c r="B25" s="1" t="s">
-        <v>21</v>
+        <v>32</v>
       </c>
       <c r="C25" s="2">
-        <v>45855</v>
+        <v>62562</v>
       </c>
       <c r="D25" s="2">
-        <v>26628</v>
+        <v>39597</v>
       </c>
       <c r="E25" s="5">
-        <v>19227</v>
+        <v>22965</v>
       </c>
       <c r="F25" s="7" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="G25" s="2"/>
       <c r="H25" s="2"/>
@@ -944,52 +956,52 @@
     </row>
     <row r="26" ht="30" customHeight="1">
       <c r="A26" s="1" t="s">
-        <v>6</v>
+        <v>36</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="C26" s="2">
-        <v>27114</v>
+        <v>90259</v>
       </c>
       <c r="D26" s="2">
-        <v>48410</v>
-      </c>
-      <c r="E26" s="3">
-        <v>-21296</v>
-      </c>
-      <c r="F26" s="4" t="s">
-        <v>33</v>
+        <v>47163</v>
+      </c>
+      <c r="E26" s="5">
+        <v>43096</v>
+      </c>
+      <c r="F26" s="7" t="s">
+        <v>37</v>
       </c>
       <c r="G26" s="2">
-        <v>180909</v>
+        <v>229134</v>
       </c>
       <c r="H26" s="2">
-        <v>118999</v>
+        <v>104815</v>
       </c>
       <c r="I26" s="5">
-        <v>61910</v>
+        <v>124319</v>
       </c>
       <c r="J26" s="8">
-        <v>8.749999999999998</v>
+        <v>52.75</v>
       </c>
     </row>
     <row r="27" ht="30" customHeight="1">
       <c r="A27" s="1"/>
       <c r="B27" s="1" t="s">
-        <v>21</v>
+        <v>3</v>
       </c>
       <c r="C27" s="2">
-        <v>93297</v>
+        <v>62601</v>
       </c>
       <c r="D27" s="2">
-        <v>36960</v>
+        <v>48592</v>
       </c>
       <c r="E27" s="5">
-        <v>56337</v>
+        <v>14009</v>
       </c>
       <c r="F27" s="7" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="G27" s="2"/>
       <c r="H27" s="2"/>
@@ -999,19 +1011,19 @@
     <row r="28" ht="30" customHeight="1">
       <c r="A28" s="1"/>
       <c r="B28" s="1" t="s">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="C28" s="2">
-        <v>60498</v>
+        <v>76274</v>
       </c>
       <c r="D28" s="2">
-        <v>33629</v>
+        <v>9060</v>
       </c>
       <c r="E28" s="5">
-        <v>26869</v>
+        <v>67214</v>
       </c>
       <c r="F28" s="7" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="G28" s="2"/>
       <c r="H28" s="2"/>
@@ -1020,52 +1032,52 @@
     </row>
     <row r="29" ht="30" customHeight="1">
       <c r="A29" s="1" t="s">
-        <v>11</v>
+        <v>31</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C29" s="2">
-        <v>69704</v>
+        <v>46704</v>
       </c>
       <c r="D29" s="2">
-        <v>45718</v>
+        <v>33154</v>
       </c>
       <c r="E29" s="5">
-        <v>23986</v>
+        <v>13550</v>
       </c>
       <c r="F29" s="7" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="G29" s="2">
-        <v>151085</v>
+        <v>230267</v>
       </c>
       <c r="H29" s="2">
-        <v>87765</v>
+        <v>60209</v>
       </c>
       <c r="I29" s="5">
-        <v>63320</v>
+        <v>170058</v>
       </c>
       <c r="J29" s="8">
-        <v>40.43666666666667</v>
+        <v>66.36666666666667</v>
       </c>
     </row>
     <row r="30" ht="30" customHeight="1">
       <c r="A30" s="1"/>
       <c r="B30" s="1" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="C30" s="2">
-        <v>20102</v>
+        <v>89209</v>
       </c>
       <c r="D30" s="2">
-        <v>13308</v>
+        <v>20267</v>
       </c>
       <c r="E30" s="5">
-        <v>6794</v>
+        <v>68942</v>
       </c>
       <c r="F30" s="7" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="G30" s="2"/>
       <c r="H30" s="2"/>
@@ -1075,19 +1087,19 @@
     <row r="31" ht="30" customHeight="1">
       <c r="A31" s="1"/>
       <c r="B31" s="1" t="s">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="C31" s="2">
-        <v>61279</v>
+        <v>94354</v>
       </c>
       <c r="D31" s="2">
-        <v>28739</v>
+        <v>6788</v>
       </c>
       <c r="E31" s="5">
-        <v>32540</v>
+        <v>87566</v>
       </c>
       <c r="F31" s="7" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="G31" s="2"/>
       <c r="H31" s="2"/>
@@ -1096,16 +1108,16 @@
     </row>
     <row r="32" ht="30" customHeight="1">
       <c r="G32" s="10">
-        <v>1794400</v>
+        <v>1853327</v>
       </c>
       <c r="H32" s="10">
-        <v>919587</v>
+        <v>868927</v>
       </c>
       <c r="I32" s="12">
-        <v>874813</v>
+        <v>984400</v>
       </c>
       <c r="J32" s="13">
-        <v>34.998000000000005</v>
+        <v>33.385666666666665</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs(core): refresh generated example workbooks
</commit_message>
<xml_diff>
--- a/packages/typed-xlsx/examples/financial-report-stream.xlsx
+++ b/packages/typed-xlsx/examples/financial-report-stream.xlsx
@@ -8,135 +8,126 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="43">
-  <si>
-    <t>2023-12</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="40">
+  <si>
+    <t>2023-08</t>
+  </si>
+  <si>
+    <t>R&amp;D</t>
+  </si>
+  <si>
+    <t>-20.14%</t>
+  </si>
+  <si>
+    <t>Sales</t>
+  </si>
+  <si>
+    <t>44.41%</t>
+  </si>
+  <si>
+    <t>-7.59%</t>
+  </si>
+  <si>
+    <t>2023-04</t>
+  </si>
+  <si>
+    <t>73.64%</t>
+  </si>
+  <si>
+    <t>Human Resources</t>
+  </si>
+  <si>
+    <t>43.95%</t>
+  </si>
+  <si>
+    <t>87.75%</t>
+  </si>
+  <si>
+    <t>Marketing</t>
+  </si>
+  <si>
+    <t>66.78%</t>
+  </si>
+  <si>
+    <t>53.55%</t>
   </si>
   <si>
     <t>Customer Support</t>
   </si>
   <si>
-    <t>-310.19%</t>
-  </si>
-  <si>
-    <t>R&amp;D</t>
-  </si>
-  <si>
-    <t>46.65%</t>
-  </si>
-  <si>
-    <t>Marketing</t>
-  </si>
-  <si>
-    <t>73.2%</t>
-  </si>
-  <si>
-    <t>2023-09</t>
-  </si>
-  <si>
-    <t>70.63%</t>
-  </si>
-  <si>
-    <t>-37.95%</t>
-  </si>
-  <si>
-    <t>50.77%</t>
-  </si>
-  <si>
-    <t>2023-03</t>
-  </si>
-  <si>
-    <t>36.12%</t>
-  </si>
-  <si>
-    <t>Human Resources</t>
-  </si>
-  <si>
-    <t>89.12%</t>
-  </si>
-  <si>
-    <t>-34.95%</t>
+    <t>-105.19%</t>
   </si>
   <si>
     <t>2023-11</t>
   </si>
   <si>
-    <t>91.28%</t>
-  </si>
-  <si>
-    <t>53.04%</t>
-  </si>
-  <si>
-    <t>14.21%</t>
-  </si>
-  <si>
-    <t>-46.19%</t>
-  </si>
-  <si>
-    <t>70.19%</t>
-  </si>
-  <si>
-    <t>63.49%</t>
-  </si>
-  <si>
-    <t>2023-04</t>
-  </si>
-  <si>
-    <t>17.85%</t>
-  </si>
-  <si>
-    <t>29.76%</t>
-  </si>
-  <si>
-    <t>85.11%</t>
-  </si>
-  <si>
-    <t>2023-02</t>
-  </si>
-  <si>
-    <t>53.94%</t>
-  </si>
-  <si>
-    <t>26.94%</t>
-  </si>
-  <si>
-    <t>8.78%</t>
-  </si>
-  <si>
-    <t>2023-01</t>
-  </si>
-  <si>
-    <t>Sales</t>
-  </si>
-  <si>
-    <t>64.4%</t>
-  </si>
-  <si>
-    <t>91.31%</t>
-  </si>
-  <si>
-    <t>36.71%</t>
+    <t>56.73%</t>
+  </si>
+  <si>
+    <t>-40.36%</t>
+  </si>
+  <si>
+    <t>67.89%</t>
+  </si>
+  <si>
+    <t>41.37%</t>
+  </si>
+  <si>
+    <t>82.22%</t>
+  </si>
+  <si>
+    <t>34.29%</t>
+  </si>
+  <si>
+    <t>75.77%</t>
+  </si>
+  <si>
+    <t>24.14%</t>
+  </si>
+  <si>
+    <t>58.13%</t>
+  </si>
+  <si>
+    <t>-7.77%</t>
+  </si>
+  <si>
+    <t>43.97%</t>
+  </si>
+  <si>
+    <t>56.56%</t>
+  </si>
+  <si>
+    <t>78.2%</t>
+  </si>
+  <si>
+    <t>63.6%</t>
+  </si>
+  <si>
+    <t>78.48%</t>
   </si>
   <si>
     <t>2023-07</t>
   </si>
   <si>
-    <t>47.75%</t>
-  </si>
-  <si>
-    <t>22.38%</t>
-  </si>
-  <si>
-    <t>88.12%</t>
-  </si>
-  <si>
-    <t>29.01%</t>
-  </si>
-  <si>
-    <t>77.28%</t>
-  </si>
-  <si>
-    <t>92.81%</t>
+    <t>74.03%</t>
+  </si>
+  <si>
+    <t>82.79%</t>
+  </si>
+  <si>
+    <t>37.81%</t>
+  </si>
+  <si>
+    <t>2023-06</t>
+  </si>
+  <si>
+    <t>-62.42%</t>
+  </si>
+  <si>
+    <t>-123.9%</t>
+  </si>
+  <si>
+    <t>72.8%</t>
   </si>
 </sst>
 </file>
@@ -245,13 +236,13 @@
     <xf numFmtId="164" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -354,28 +345,28 @@
         <v>1</v>
       </c>
       <c r="C2" s="2">
-        <v>11020</v>
+        <v>24842</v>
       </c>
       <c r="D2" s="2">
-        <v>45203</v>
+        <v>29846</v>
       </c>
       <c r="E2" s="3">
-        <v>-34183</v>
+        <v>-5004</v>
       </c>
       <c r="F2" s="4" t="s">
         <v>2</v>
       </c>
       <c r="G2" s="2">
-        <v>146693</v>
+        <v>137503</v>
       </c>
       <c r="H2" s="2">
-        <v>93690</v>
+        <v>115274</v>
       </c>
       <c r="I2" s="5">
-        <v>53003</v>
+        <v>22229</v>
       </c>
       <c r="J2" s="6">
-        <v>-63.44666666666668</v>
+        <v>5.559999999999999</v>
       </c>
     </row>
     <row r="3" ht="30" customHeight="1">
@@ -384,13 +375,13 @@
         <v>3</v>
       </c>
       <c r="C3" s="2">
-        <v>45676</v>
+        <v>68812</v>
       </c>
       <c r="D3" s="2">
-        <v>24369</v>
+        <v>38252</v>
       </c>
       <c r="E3" s="5">
-        <v>21307</v>
+        <v>30560</v>
       </c>
       <c r="F3" s="7" t="s">
         <v>4</v>
@@ -403,19 +394,19 @@
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="1"/>
       <c r="B4" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C4" s="2">
+        <v>43849</v>
+      </c>
+      <c r="D4" s="2">
+        <v>47176</v>
+      </c>
+      <c r="E4" s="3">
+        <v>-3327</v>
+      </c>
+      <c r="F4" s="4" t="s">
         <v>5</v>
-      </c>
-      <c r="C4" s="2">
-        <v>89997</v>
-      </c>
-      <c r="D4" s="2">
-        <v>24118</v>
-      </c>
-      <c r="E4" s="5">
-        <v>65879</v>
-      </c>
-      <c r="F4" s="7" t="s">
-        <v>6</v>
       </c>
       <c r="G4" s="2"/>
       <c r="H4" s="2"/>
@@ -424,71 +415,71 @@
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C5" s="2">
+        <v>63197</v>
+      </c>
+      <c r="D5" s="2">
+        <v>16661</v>
+      </c>
+      <c r="E5" s="5">
+        <v>46536</v>
+      </c>
+      <c r="F5" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C5" s="2">
-        <v>35786</v>
-      </c>
-      <c r="D5" s="2">
-        <v>10510</v>
-      </c>
-      <c r="E5" s="5">
-        <v>25276</v>
-      </c>
-      <c r="F5" s="7" t="s">
-        <v>8</v>
-      </c>
       <c r="G5" s="2">
-        <v>94558</v>
+        <v>219760</v>
       </c>
       <c r="H5" s="2">
-        <v>56561</v>
+        <v>60668</v>
       </c>
       <c r="I5" s="5">
-        <v>37997</v>
-      </c>
-      <c r="J5" s="8">
-        <v>27.816666666666663</v>
+        <v>159092</v>
+      </c>
+      <c r="J5" s="6">
+        <v>68.44666666666667</v>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="1"/>
       <c r="B6" s="1" t="s">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="C6" s="2">
-        <v>19296</v>
+        <v>56690</v>
       </c>
       <c r="D6" s="2">
-        <v>26618</v>
-      </c>
-      <c r="E6" s="3">
-        <v>-7322</v>
-      </c>
-      <c r="F6" s="4" t="s">
+        <v>31775</v>
+      </c>
+      <c r="E6" s="5">
+        <v>24915</v>
+      </c>
+      <c r="F6" s="7" t="s">
         <v>9</v>
       </c>
       <c r="G6" s="2"/>
       <c r="H6" s="2"/>
       <c r="I6" s="5"/>
-      <c r="J6" s="8"/>
+      <c r="J6" s="6"/>
     </row>
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="1"/>
       <c r="B7" s="1" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C7" s="2">
-        <v>39476</v>
+        <v>99873</v>
       </c>
       <c r="D7" s="2">
-        <v>19433</v>
+        <v>12232</v>
       </c>
       <c r="E7" s="5">
-        <v>20043</v>
+        <v>87641</v>
       </c>
       <c r="F7" s="7" t="s">
         <v>10</v>
@@ -496,75 +487,75 @@
       <c r="G7" s="2"/>
       <c r="H7" s="2"/>
       <c r="I7" s="5"/>
-      <c r="J7" s="8"/>
+      <c r="J7" s="6"/>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B8" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B8" s="1" t="s">
-        <v>5</v>
-      </c>
       <c r="C8" s="2">
-        <v>15519</v>
+        <v>28837</v>
       </c>
       <c r="D8" s="2">
-        <v>9914</v>
+        <v>9581</v>
       </c>
       <c r="E8" s="5">
-        <v>5605</v>
+        <v>19256</v>
       </c>
       <c r="F8" s="7" t="s">
         <v>12</v>
       </c>
       <c r="G8" s="2">
-        <v>121042</v>
+        <v>93124</v>
       </c>
       <c r="H8" s="2">
-        <v>63386</v>
+        <v>72127</v>
       </c>
       <c r="I8" s="5">
-        <v>57656</v>
-      </c>
-      <c r="J8" s="8">
-        <v>30.096666666666668</v>
+        <v>20997</v>
+      </c>
+      <c r="J8" s="6">
+        <v>5.046666666666667</v>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="1"/>
       <c r="B9" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C9" s="2">
+        <v>43698</v>
+      </c>
+      <c r="D9" s="2">
+        <v>20299</v>
+      </c>
+      <c r="E9" s="5">
+        <v>23399</v>
+      </c>
+      <c r="F9" s="7" t="s">
         <v>13</v>
-      </c>
-      <c r="C9" s="2">
-        <v>71676</v>
-      </c>
-      <c r="D9" s="2">
-        <v>7797</v>
-      </c>
-      <c r="E9" s="5">
-        <v>63879</v>
-      </c>
-      <c r="F9" s="7" t="s">
-        <v>14</v>
       </c>
       <c r="G9" s="2"/>
       <c r="H9" s="2"/>
       <c r="I9" s="5"/>
-      <c r="J9" s="8"/>
+      <c r="J9" s="6"/>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="1"/>
       <c r="B10" s="1" t="s">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="C10" s="2">
-        <v>33847</v>
+        <v>20589</v>
       </c>
       <c r="D10" s="2">
-        <v>45675</v>
+        <v>42247</v>
       </c>
       <c r="E10" s="3">
-        <v>-11828</v>
+        <v>-21658</v>
       </c>
       <c r="F10" s="4" t="s">
         <v>15</v>
@@ -572,75 +563,75 @@
       <c r="G10" s="2"/>
       <c r="H10" s="2"/>
       <c r="I10" s="5"/>
-      <c r="J10" s="8"/>
+      <c r="J10" s="6"/>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="1" t="s">
         <v>16</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C11" s="2">
-        <v>83517</v>
+        <v>45084</v>
       </c>
       <c r="D11" s="2">
-        <v>7285</v>
+        <v>19508</v>
       </c>
       <c r="E11" s="5">
-        <v>76232</v>
+        <v>25576</v>
       </c>
       <c r="F11" s="7" t="s">
         <v>17</v>
       </c>
       <c r="G11" s="2">
-        <v>218949</v>
+        <v>131824</v>
       </c>
       <c r="H11" s="2">
-        <v>88432</v>
+        <v>78039</v>
       </c>
       <c r="I11" s="5">
-        <v>130517</v>
-      </c>
-      <c r="J11" s="8">
-        <v>52.843333333333334</v>
+        <v>53785</v>
+      </c>
+      <c r="J11" s="6">
+        <v>28.086666666666662</v>
       </c>
     </row>
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="1"/>
       <c r="B12" s="1" t="s">
-        <v>3</v>
+        <v>14</v>
       </c>
       <c r="C12" s="2">
-        <v>90250</v>
+        <v>28343</v>
       </c>
       <c r="D12" s="2">
-        <v>42384</v>
-      </c>
-      <c r="E12" s="5">
-        <v>47866</v>
-      </c>
-      <c r="F12" s="7" t="s">
+        <v>39781</v>
+      </c>
+      <c r="E12" s="3">
+        <v>-11438</v>
+      </c>
+      <c r="F12" s="4" t="s">
         <v>18</v>
       </c>
       <c r="G12" s="2"/>
       <c r="H12" s="2"/>
       <c r="I12" s="5"/>
-      <c r="J12" s="8"/>
+      <c r="J12" s="6"/>
     </row>
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="1"/>
       <c r="B13" s="1" t="s">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="C13" s="2">
-        <v>45182</v>
+        <v>58397</v>
       </c>
       <c r="D13" s="2">
-        <v>38763</v>
+        <v>18750</v>
       </c>
       <c r="E13" s="5">
-        <v>6419</v>
+        <v>39647</v>
       </c>
       <c r="F13" s="7" t="s">
         <v>19</v>
@@ -648,53 +639,53 @@
       <c r="G13" s="2"/>
       <c r="H13" s="2"/>
       <c r="I13" s="5"/>
-      <c r="J13" s="8"/>
+      <c r="J13" s="6"/>
     </row>
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="1" t="s">
         <v>16</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="C14" s="2">
-        <v>25010</v>
+        <v>63623</v>
       </c>
       <c r="D14" s="2">
-        <v>36562</v>
-      </c>
-      <c r="E14" s="3">
-        <v>-11552</v>
-      </c>
-      <c r="F14" s="4" t="s">
+        <v>37301</v>
+      </c>
+      <c r="E14" s="5">
+        <v>26322</v>
+      </c>
+      <c r="F14" s="7" t="s">
         <v>20</v>
       </c>
       <c r="G14" s="2">
-        <v>169731</v>
+        <v>224194</v>
       </c>
       <c r="H14" s="2">
-        <v>85448</v>
+        <v>97094</v>
       </c>
       <c r="I14" s="5">
-        <v>84283</v>
-      </c>
-      <c r="J14" s="8">
-        <v>29.163333333333338</v>
+        <v>127100</v>
+      </c>
+      <c r="J14" s="6">
+        <v>52.626666666666665</v>
       </c>
     </row>
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="1"/>
       <c r="B15" s="1" t="s">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="C15" s="2">
-        <v>58889</v>
+        <v>95388</v>
       </c>
       <c r="D15" s="2">
-        <v>17553</v>
+        <v>16959</v>
       </c>
       <c r="E15" s="5">
-        <v>41336</v>
+        <v>78429</v>
       </c>
       <c r="F15" s="7" t="s">
         <v>21</v>
@@ -702,21 +693,21 @@
       <c r="G15" s="2"/>
       <c r="H15" s="2"/>
       <c r="I15" s="5"/>
-      <c r="J15" s="8"/>
+      <c r="J15" s="6"/>
     </row>
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="1"/>
       <c r="B16" s="1" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C16" s="2">
-        <v>85832</v>
+        <v>65183</v>
       </c>
       <c r="D16" s="2">
-        <v>31333</v>
+        <v>42834</v>
       </c>
       <c r="E16" s="5">
-        <v>54499</v>
+        <v>22349</v>
       </c>
       <c r="F16" s="7" t="s">
         <v>22</v>
@@ -724,137 +715,137 @@
       <c r="G16" s="2"/>
       <c r="H16" s="2"/>
       <c r="I16" s="5"/>
-      <c r="J16" s="8"/>
+      <c r="J16" s="6"/>
     </row>
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C17" s="2">
+        <v>99449</v>
+      </c>
+      <c r="D17" s="2">
+        <v>24095</v>
+      </c>
+      <c r="E17" s="5">
+        <v>75354</v>
+      </c>
+      <c r="F17" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="B17" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C17" s="2">
-        <v>59271</v>
-      </c>
-      <c r="D17" s="2">
-        <v>48689</v>
-      </c>
-      <c r="E17" s="5">
-        <v>10582</v>
-      </c>
-      <c r="F17" s="7" t="s">
-        <v>24</v>
-      </c>
       <c r="G17" s="2">
-        <v>188391</v>
+        <v>241339</v>
       </c>
       <c r="H17" s="2">
-        <v>100311</v>
+        <v>98944</v>
       </c>
       <c r="I17" s="5">
-        <v>88080</v>
-      </c>
-      <c r="J17" s="8">
-        <v>44.24</v>
+        <v>142395</v>
+      </c>
+      <c r="J17" s="6">
+        <v>52.68</v>
       </c>
     </row>
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="1"/>
       <c r="B18" s="1" t="s">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="C18" s="2">
-        <v>58526</v>
+        <v>45432</v>
       </c>
       <c r="D18" s="2">
-        <v>41111</v>
+        <v>34466</v>
       </c>
       <c r="E18" s="5">
-        <v>17415</v>
+        <v>10966</v>
       </c>
       <c r="F18" s="7" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="G18" s="2"/>
       <c r="H18" s="2"/>
       <c r="I18" s="5"/>
-      <c r="J18" s="8"/>
+      <c r="J18" s="6"/>
     </row>
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="1"/>
       <c r="B19" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C19" s="2">
-        <v>70594</v>
+        <v>96458</v>
       </c>
       <c r="D19" s="2">
-        <v>10511</v>
+        <v>40383</v>
       </c>
       <c r="E19" s="5">
-        <v>60083</v>
+        <v>56075</v>
       </c>
       <c r="F19" s="7" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G19" s="2"/>
       <c r="H19" s="2"/>
       <c r="I19" s="5"/>
-      <c r="J19" s="8"/>
+      <c r="J19" s="6"/>
     </row>
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="1" t="s">
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C20" s="2">
-        <v>98904</v>
+        <v>44248</v>
       </c>
       <c r="D20" s="2">
-        <v>45553</v>
-      </c>
-      <c r="E20" s="5">
-        <v>53351</v>
-      </c>
-      <c r="F20" s="7" t="s">
-        <v>28</v>
+        <v>47685</v>
+      </c>
+      <c r="E20" s="3">
+        <v>-3437</v>
+      </c>
+      <c r="F20" s="4" t="s">
+        <v>26</v>
       </c>
       <c r="G20" s="2">
-        <v>209634</v>
+        <v>185682</v>
       </c>
       <c r="H20" s="2">
-        <v>134807</v>
+        <v>118637</v>
       </c>
       <c r="I20" s="5">
-        <v>74827</v>
-      </c>
-      <c r="J20" s="8">
-        <v>29.886666666666667</v>
+        <v>67045</v>
+      </c>
+      <c r="J20" s="6">
+        <v>30.92</v>
       </c>
     </row>
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="1"/>
       <c r="B21" s="1" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="C21" s="2">
-        <v>64724</v>
+        <v>75572</v>
       </c>
       <c r="D21" s="2">
-        <v>47288</v>
+        <v>42341</v>
       </c>
       <c r="E21" s="5">
-        <v>17436</v>
+        <v>33231</v>
       </c>
       <c r="F21" s="7" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="G21" s="2"/>
       <c r="H21" s="2"/>
       <c r="I21" s="5"/>
-      <c r="J21" s="8"/>
+      <c r="J21" s="6"/>
     </row>
     <row r="22" ht="30" customHeight="1">
       <c r="A22" s="1"/>
@@ -862,222 +853,222 @@
         <v>3</v>
       </c>
       <c r="C22" s="2">
-        <v>46006</v>
+        <v>65862</v>
       </c>
       <c r="D22" s="2">
-        <v>41966</v>
+        <v>28611</v>
       </c>
       <c r="E22" s="5">
-        <v>4040</v>
+        <v>37251</v>
       </c>
       <c r="F22" s="7" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="G22" s="2"/>
       <c r="H22" s="2"/>
       <c r="I22" s="5"/>
-      <c r="J22" s="8"/>
+      <c r="J22" s="6"/>
     </row>
     <row r="23" ht="30" customHeight="1">
       <c r="A23" s="1" t="s">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>32</v>
+        <v>3</v>
       </c>
       <c r="C23" s="2">
-        <v>95945</v>
+        <v>69746</v>
       </c>
       <c r="D23" s="2">
-        <v>34159</v>
+        <v>15203</v>
       </c>
       <c r="E23" s="5">
-        <v>61786</v>
+        <v>54543</v>
       </c>
       <c r="F23" s="7" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="G23" s="2">
-        <v>244928</v>
+        <v>239669</v>
       </c>
       <c r="H23" s="2">
-        <v>81268</v>
+        <v>65026</v>
       </c>
       <c r="I23" s="5">
-        <v>163660</v>
-      </c>
-      <c r="J23" s="8">
-        <v>64.14</v>
+        <v>174643</v>
+      </c>
+      <c r="J23" s="6">
+        <v>73.42666666666668</v>
       </c>
     </row>
     <row r="24" ht="30" customHeight="1">
       <c r="A24" s="1"/>
       <c r="B24" s="1" t="s">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="C24" s="2">
-        <v>86421</v>
+        <v>89099</v>
       </c>
       <c r="D24" s="2">
-        <v>7512</v>
+        <v>32431</v>
       </c>
       <c r="E24" s="5">
-        <v>78909</v>
+        <v>56668</v>
       </c>
       <c r="F24" s="7" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="G24" s="2"/>
       <c r="H24" s="2"/>
       <c r="I24" s="5"/>
-      <c r="J24" s="8"/>
+      <c r="J24" s="6"/>
     </row>
     <row r="25" ht="30" customHeight="1">
       <c r="A25" s="1"/>
       <c r="B25" s="1" t="s">
-        <v>32</v>
+        <v>1</v>
       </c>
       <c r="C25" s="2">
-        <v>62562</v>
+        <v>80824</v>
       </c>
       <c r="D25" s="2">
-        <v>39597</v>
+        <v>17392</v>
       </c>
       <c r="E25" s="5">
-        <v>22965</v>
+        <v>63432</v>
       </c>
       <c r="F25" s="7" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="G25" s="2"/>
       <c r="H25" s="2"/>
       <c r="I25" s="5"/>
-      <c r="J25" s="8"/>
+      <c r="J25" s="6"/>
     </row>
     <row r="26" ht="30" customHeight="1">
       <c r="A26" s="1" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="C26" s="2">
-        <v>90259</v>
+        <v>35971</v>
       </c>
       <c r="D26" s="2">
-        <v>47163</v>
+        <v>9340</v>
       </c>
       <c r="E26" s="5">
-        <v>43096</v>
+        <v>26631</v>
       </c>
       <c r="F26" s="7" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="G26" s="2">
-        <v>229134</v>
+        <v>164895</v>
       </c>
       <c r="H26" s="2">
-        <v>104815</v>
+        <v>58749</v>
       </c>
       <c r="I26" s="5">
-        <v>124319</v>
-      </c>
-      <c r="J26" s="8">
-        <v>52.75</v>
+        <v>106146</v>
+      </c>
+      <c r="J26" s="6">
+        <v>64.87666666666667</v>
       </c>
     </row>
     <row r="27" ht="30" customHeight="1">
       <c r="A27" s="1"/>
       <c r="B27" s="1" t="s">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="C27" s="2">
-        <v>62601</v>
+        <v>68412</v>
       </c>
       <c r="D27" s="2">
-        <v>48592</v>
+        <v>11774</v>
       </c>
       <c r="E27" s="5">
-        <v>14009</v>
+        <v>56638</v>
       </c>
       <c r="F27" s="7" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="G27" s="2"/>
       <c r="H27" s="2"/>
       <c r="I27" s="5"/>
-      <c r="J27" s="8"/>
+      <c r="J27" s="6"/>
     </row>
     <row r="28" ht="30" customHeight="1">
       <c r="A28" s="1"/>
       <c r="B28" s="1" t="s">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="C28" s="2">
-        <v>76274</v>
+        <v>60512</v>
       </c>
       <c r="D28" s="2">
-        <v>9060</v>
+        <v>37635</v>
       </c>
       <c r="E28" s="5">
-        <v>67214</v>
+        <v>22877</v>
       </c>
       <c r="F28" s="7" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="G28" s="2"/>
       <c r="H28" s="2"/>
       <c r="I28" s="5"/>
-      <c r="J28" s="8"/>
+      <c r="J28" s="6"/>
     </row>
     <row r="29" ht="30" customHeight="1">
       <c r="A29" s="1" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C29" s="2">
-        <v>46704</v>
+        <v>22859</v>
       </c>
       <c r="D29" s="2">
-        <v>33154</v>
-      </c>
-      <c r="E29" s="5">
-        <v>13550</v>
-      </c>
-      <c r="F29" s="7" t="s">
-        <v>40</v>
+        <v>37128</v>
+      </c>
+      <c r="E29" s="3">
+        <v>-14269</v>
+      </c>
+      <c r="F29" s="4" t="s">
+        <v>37</v>
       </c>
       <c r="G29" s="2">
-        <v>230267</v>
+        <v>126249</v>
       </c>
       <c r="H29" s="2">
-        <v>60209</v>
+        <v>99646</v>
       </c>
       <c r="I29" s="5">
-        <v>170058</v>
+        <v>26603</v>
       </c>
       <c r="J29" s="8">
-        <v>66.36666666666667</v>
+        <v>-37.839999999999996</v>
       </c>
     </row>
     <row r="30" ht="30" customHeight="1">
       <c r="A30" s="1"/>
       <c r="B30" s="1" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C30" s="2">
-        <v>89209</v>
+        <v>17486</v>
       </c>
       <c r="D30" s="2">
-        <v>20267</v>
-      </c>
-      <c r="E30" s="5">
-        <v>68942</v>
-      </c>
-      <c r="F30" s="7" t="s">
-        <v>41</v>
+        <v>39152</v>
+      </c>
+      <c r="E30" s="3">
+        <v>-21666</v>
+      </c>
+      <c r="F30" s="4" t="s">
+        <v>38</v>
       </c>
       <c r="G30" s="2"/>
       <c r="H30" s="2"/>
@@ -1087,19 +1078,19 @@
     <row r="31" ht="30" customHeight="1">
       <c r="A31" s="1"/>
       <c r="B31" s="1" t="s">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="C31" s="2">
-        <v>94354</v>
+        <v>85904</v>
       </c>
       <c r="D31" s="2">
-        <v>6788</v>
+        <v>23366</v>
       </c>
       <c r="E31" s="5">
-        <v>87566</v>
+        <v>62538</v>
       </c>
       <c r="F31" s="7" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G31" s="2"/>
       <c r="H31" s="2"/>
@@ -1108,16 +1099,16 @@
     </row>
     <row r="32" ht="30" customHeight="1">
       <c r="G32" s="10">
-        <v>1853327</v>
+        <v>1764239</v>
       </c>
       <c r="H32" s="10">
-        <v>868927</v>
+        <v>864204</v>
       </c>
       <c r="I32" s="12">
-        <v>984400</v>
+        <v>900035</v>
       </c>
       <c r="J32" s="13">
-        <v>33.385666666666665</v>
+        <v>34.383</v>
       </c>
     </row>
   </sheetData>

</xml_diff>